<commit_message>
attendance and other updtes
</commit_message>
<xml_diff>
--- a/assets/misc/2026/2026_Attendance.xlsx
+++ b/assets/misc/2026/2026_Attendance.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Documents\git\sqlsatwebsite\assets\misc\2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2EAE2CA-1540-470A-AC36-A41872D3AC98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{054AC06E-9201-4BD6-9BC0-C5AEA7B3676E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15990" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2190" yWindow="45" windowWidth="22995" windowHeight="15165" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Attendance" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="41">
   <si>
     <t>Date</t>
   </si>
@@ -151,6 +151,12 @@
   </si>
   <si>
     <t>Day of Data PNW 2026 (#1149)</t>
+  </si>
+  <si>
+    <t>Day of Data Detroit 2026 (#1164)</t>
+  </si>
+  <si>
+    <t>Day of Data Vitória 2026 (#1156)</t>
   </si>
 </sst>
 </file>
@@ -239,7 +245,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -298,6 +304,8 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1"/>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Comma" xfId="2" builtinId="3"/>
@@ -605,7 +613,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:I33"/>
+  <dimension ref="A1:I35"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.7109375" style="10" bestFit="1" customWidth="1"/>
@@ -659,7 +667,7 @@
         <v>108</v>
       </c>
       <c r="E2" s="7">
-        <f t="shared" ref="E2:E26" si="0">IF(C2=0,0,+(C2-D2)/C2)</f>
+        <f t="shared" ref="E2:E28" si="0">IF(C2=0,0,+(C2-D2)/C2)</f>
         <v>0.63758389261744963</v>
       </c>
     </row>
@@ -962,14 +970,14 @@
         <v>33</v>
       </c>
       <c r="C19" s="6">
-        <v>0</v>
+        <v>128</v>
       </c>
       <c r="D19" s="6">
-        <v>0</v>
+        <v>116</v>
       </c>
       <c r="E19" s="7">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>9.375E-2</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -991,47 +999,47 @@
       </c>
     </row>
     <row r="21" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="10">
+      <c r="A21" s="5">
+        <v>46277</v>
+      </c>
+      <c r="B21" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="C21" s="6">
+        <v>0</v>
+      </c>
+      <c r="D21" s="6">
+        <v>0</v>
+      </c>
+      <c r="E21" s="7">
+        <f t="shared" ref="E21" si="1">IF(C21=0,0,+(C21-D21)/C21)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="10">
         <v>46284</v>
       </c>
-      <c r="B21" s="12" t="s">
+      <c r="B22" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="C21" s="6">
-        <v>0</v>
-      </c>
-      <c r="D21" s="6">
-        <v>0</v>
-      </c>
-      <c r="E21" s="7">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="5">
-        <v>46298</v>
-      </c>
-      <c r="B22" s="12" t="s">
-        <v>35</v>
-      </c>
       <c r="C22" s="6">
-        <v>0</v>
+        <v>140</v>
       </c>
       <c r="D22" s="6">
-        <v>0</v>
+        <v>65</v>
       </c>
       <c r="E22" s="7">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.5357142857142857</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="5">
-        <v>46319</v>
+      <c r="A23" s="10">
+        <v>46284</v>
       </c>
       <c r="B23" s="12" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C23" s="6">
         <v>0</v>
@@ -1040,16 +1048,16 @@
         <v>0</v>
       </c>
       <c r="E23" s="7">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="E23" si="2">IF(C23=0,0,+(C23-D23)/C23)</f>
         <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="5">
-        <v>46319</v>
+        <v>46298</v>
       </c>
       <c r="B24" s="12" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C24" s="6">
         <v>0</v>
@@ -1064,48 +1072,74 @@
     </row>
     <row r="25" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="5">
+        <v>46319</v>
+      </c>
+      <c r="B25" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="C25" s="6">
+        <v>0</v>
+      </c>
+      <c r="D25" s="6">
+        <v>0</v>
+      </c>
+      <c r="E25" s="7">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="5">
+        <v>46319</v>
+      </c>
+      <c r="B26" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="C26" s="6">
+        <v>0</v>
+      </c>
+      <c r="D26" s="6">
+        <v>0</v>
+      </c>
+      <c r="E26" s="7">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="5">
         <v>46333</v>
       </c>
-      <c r="B25" s="12" t="s">
+      <c r="B27" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="C25" s="6">
-        <v>0</v>
-      </c>
-      <c r="D25" s="6">
-        <v>0</v>
-      </c>
-      <c r="E25" s="7">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="5"/>
-      <c r="B26" s="12"/>
-      <c r="E26" s="7">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="5"/>
-      <c r="B27" s="12"/>
-      <c r="E27" s="7"/>
+      <c r="C27" s="6">
+        <v>0</v>
+      </c>
+      <c r="D27" s="6">
+        <v>0</v>
+      </c>
+      <c r="E27" s="7">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="28" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="5"/>
-      <c r="B28" s="13"/>
-      <c r="E28" s="7"/>
-    </row>
-    <row r="29" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B28" s="12"/>
+      <c r="E28" s="7">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="5"/>
-      <c r="B29" s="9"/>
+      <c r="B29" s="12"/>
       <c r="E29" s="7"/>
     </row>
     <row r="30" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="5"/>
-      <c r="B30" s="9"/>
+      <c r="B30" s="13"/>
       <c r="E30" s="7"/>
     </row>
     <row r="31" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1123,9 +1157,19 @@
       <c r="B33" s="9"/>
       <c r="E33" s="7"/>
     </row>
+    <row r="34" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="5"/>
+      <c r="B34" s="9"/>
+      <c r="E34" s="7"/>
+    </row>
+    <row r="35" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="5"/>
+      <c r="B35" s="9"/>
+      <c r="E35" s="7"/>
+    </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I34">
-    <sortCondition ref="A2:A34"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I36">
+    <sortCondition ref="A2:A36"/>
   </sortState>
   <hyperlinks>
     <hyperlink ref="B2" r:id="rId1" display="https://sqlsaturday.com/2026-01-17-sqlsaturday1138/" xr:uid="{82BDF17B-780C-46C4-BDF3-6B50D2949365}"/>
@@ -1147,14 +1191,16 @@
     <hyperlink ref="B17" r:id="rId17" display="https://sqlsaturday.com/2026-06-27-sqlsaturday1154/" xr:uid="{4E193433-7FEF-42F0-9BE1-2E1B4F56DC45}"/>
     <hyperlink ref="B18" r:id="rId18" display="https://sqlsaturday.com/2026-07-18-sqlsaturday1141/" xr:uid="{B4310BB2-BE85-4D94-9531-7F04382A3C59}"/>
     <hyperlink ref="B19" r:id="rId19" display="https://sqlsaturday.com/2026-08-08-sqlsaturday1144/" xr:uid="{49013F68-7251-4303-A8A8-19F4C344B133}"/>
-    <hyperlink ref="B21" r:id="rId20" display="https://sqlsaturday.com/2026-09-19-sqlsaturday1152/" xr:uid="{1C24212F-ACFE-4FD3-A6CF-8E691EEA9C75}"/>
-    <hyperlink ref="B22" r:id="rId21" display="https://sqlsaturday.com/2026-10-03-sqlsaturday1150/" xr:uid="{80072270-983F-4E6A-AFAE-3FC24DE448B3}"/>
-    <hyperlink ref="B23" r:id="rId22" display="https://sqlsaturday.com/2026-10-24-sqlsaturday1148/" xr:uid="{111A5B01-58C6-46AB-81AC-567A7B3C8861}"/>
-    <hyperlink ref="B24" r:id="rId23" display="https://sqlsaturday.com/2026-10-24-sqlsaturday1153/" xr:uid="{29A122E2-6150-4028-BEF4-E884CED9AA91}"/>
-    <hyperlink ref="B25" r:id="rId24" display="https://sqlsaturday.com/2026-11-07-sqlsaturday1149/" xr:uid="{1C87B471-8BB8-47E8-8A2F-FEB250EAF056}"/>
+    <hyperlink ref="B22" r:id="rId20" display="https://sqlsaturday.com/2026-09-19-sqlsaturday1152/" xr:uid="{1C24212F-ACFE-4FD3-A6CF-8E691EEA9C75}"/>
+    <hyperlink ref="B24" r:id="rId21" display="https://sqlsaturday.com/2026-10-03-sqlsaturday1150/" xr:uid="{80072270-983F-4E6A-AFAE-3FC24DE448B3}"/>
+    <hyperlink ref="B25" r:id="rId22" display="https://sqlsaturday.com/2026-10-24-sqlsaturday1148/" xr:uid="{111A5B01-58C6-46AB-81AC-567A7B3C8861}"/>
+    <hyperlink ref="B26" r:id="rId23" display="https://sqlsaturday.com/2026-10-24-sqlsaturday1153/" xr:uid="{29A122E2-6150-4028-BEF4-E884CED9AA91}"/>
+    <hyperlink ref="B27" r:id="rId24" display="https://sqlsaturday.com/2026-11-07-sqlsaturday1149/" xr:uid="{1C87B471-8BB8-47E8-8A2F-FEB250EAF056}"/>
+    <hyperlink ref="B21" r:id="rId25" display="https://sqlsaturday.com/2026-09-12-sqlsaturday1164/" xr:uid="{C31C9E88-D474-46E9-9D7F-515DB0D1C4FD}"/>
+    <hyperlink ref="B23" r:id="rId26" display="https://sqlsaturday.com/2026-09-19-sqlsaturday1156/" xr:uid="{D29C5250-03B6-490D-8B76-A7A1B304D760}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId25"/>
+  <pageSetup orientation="portrait" r:id="rId27"/>
 </worksheet>
 </file>
 
@@ -1196,7 +1242,7 @@
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A2" s="10">
+      <c r="A2" s="24">
         <f>+Attendance!A2</f>
         <v>46039</v>
       </c>
@@ -1226,7 +1272,7 @@
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A3" s="10">
+      <c r="A3" s="24">
         <f>+Attendance!A3</f>
         <v>46102</v>
       </c>
@@ -1256,7 +1302,7 @@
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A4" s="10">
+      <c r="A4" s="24">
         <f>+Attendance!A4</f>
         <v>46109</v>
       </c>
@@ -1286,7 +1332,7 @@
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A5" s="10">
+      <c r="A5" s="24">
         <f>+Attendance!A5</f>
         <v>46123</v>
       </c>
@@ -1316,7 +1362,7 @@
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A6" s="10">
+      <c r="A6" s="24">
         <f>+Attendance!A6</f>
         <v>46123</v>
       </c>
@@ -1348,7 +1394,7 @@
       <c r="P6" s="23"/>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A7" s="10">
+      <c r="A7" s="24">
         <f>+Attendance!A7</f>
         <v>46130</v>
       </c>
@@ -1381,7 +1427,7 @@
       <c r="P7" s="23"/>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A8" s="10">
+      <c r="A8" s="24">
         <f>+Attendance!A8</f>
         <v>46137</v>
       </c>
@@ -1413,7 +1459,7 @@
       <c r="P8" s="22"/>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A9" s="10">
+      <c r="A9" s="24">
         <f>+Attendance!A9</f>
         <v>46137</v>
       </c>
@@ -1445,7 +1491,7 @@
       <c r="P9" s="22"/>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A10" s="10">
+      <c r="A10" s="24">
         <f>+Attendance!A10</f>
         <v>46144</v>
       </c>
@@ -1477,7 +1523,7 @@
       <c r="P10" s="22"/>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A11" s="10">
+      <c r="A11" s="24">
         <f>+Attendance!A11</f>
         <v>46158</v>
       </c>
@@ -1509,7 +1555,7 @@
       <c r="P11" s="22"/>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A12" s="10">
+      <c r="A12" s="24">
         <f>+Attendance!A12</f>
         <v>46256</v>
       </c>
@@ -1541,7 +1587,7 @@
       <c r="P12" s="22"/>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A13" s="10">
+      <c r="A13" s="24">
         <f>+Attendance!A13</f>
         <v>46165</v>
       </c>
@@ -1573,7 +1619,7 @@
       <c r="P13" s="22"/>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A14" s="10">
+      <c r="A14" s="24">
         <f>+Attendance!A14</f>
         <v>46172</v>
       </c>
@@ -1604,7 +1650,7 @@
       <c r="P14" s="22"/>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A15" s="10">
+      <c r="A15" s="24">
         <f>+Attendance!A15</f>
         <v>46186</v>
       </c>
@@ -1635,7 +1681,7 @@
       <c r="P15" s="22"/>
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A16" s="10">
+      <c r="A16" s="24">
         <f>+Attendance!A16</f>
         <v>46200</v>
       </c>
@@ -1666,7 +1712,7 @@
       <c r="P16" s="22"/>
     </row>
     <row r="17" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A17" s="10">
+      <c r="A17" s="24">
         <f>+Attendance!A17</f>
         <v>46200</v>
       </c>
@@ -1698,7 +1744,7 @@
       <c r="P17" s="22"/>
     </row>
     <row r="18" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A18" s="10">
+      <c r="A18" s="24">
         <f>+Attendance!A18</f>
         <v>46221</v>
       </c>
@@ -1730,7 +1776,7 @@
       <c r="P18" s="22"/>
     </row>
     <row r="19" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A19" s="10">
+      <c r="A19" s="24">
         <f>+Attendance!A19</f>
         <v>46242</v>
       </c>
@@ -1742,27 +1788,26 @@
         <v>0</v>
       </c>
       <c r="D19">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="E19">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F19">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="G19" s="8">
-        <f t="shared" si="3"/>
-        <v>0</v>
+        <v>61</v>
       </c>
       <c r="H19" s="8">
         <f>+Attendance!C19</f>
-        <v>0</v>
+        <v>128</v>
       </c>
       <c r="O19" s="21"/>
       <c r="P19" s="22"/>
     </row>
     <row r="20" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A20" s="10">
+      <c r="A20" s="24">
         <f>+Attendance!A20</f>
         <v>46256</v>
       </c>
@@ -1794,13 +1839,11 @@
       <c r="P20" s="22"/>
     </row>
     <row r="21" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A21" s="10">
-        <f>+Attendance!A21</f>
-        <v>46284</v>
-      </c>
-      <c r="B21" s="10" t="str">
-        <f>+Attendance!B21</f>
-        <v>Salt Lake City Day of Data 2026 (#1152)</v>
+      <c r="A21" s="25">
+        <v>46277</v>
+      </c>
+      <c r="B21" s="12" t="s">
+        <v>39</v>
       </c>
       <c r="C21">
         <v>0</v>
@@ -1816,23 +1859,21 @@
       </c>
       <c r="G21" s="8">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>140</v>
       </c>
       <c r="H21" s="8">
-        <f>+Attendance!C21</f>
-        <v>0</v>
+        <f>+Attendance!C22</f>
+        <v>140</v>
       </c>
       <c r="O21" s="21"/>
       <c r="P21" s="22"/>
     </row>
     <row r="22" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A22" s="10">
-        <f>+Attendance!A22</f>
-        <v>46298</v>
-      </c>
-      <c r="B22" s="10" t="str">
-        <f>+Attendance!B22</f>
-        <v>Boston Data and AI Saturday 2026 (#1150)</v>
+      <c r="A22" s="24">
+        <v>46284</v>
+      </c>
+      <c r="B22" s="12" t="s">
+        <v>34</v>
       </c>
       <c r="C22">
         <v>0</v>
@@ -1851,20 +1892,18 @@
         <v>0</v>
       </c>
       <c r="H22" s="8">
-        <f>+Attendance!C22</f>
+        <f>+Attendance!C24</f>
         <v>0</v>
       </c>
       <c r="O22" s="21"/>
       <c r="P22" s="22"/>
     </row>
     <row r="23" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A23" s="10">
-        <f>+Attendance!A23</f>
-        <v>46319</v>
-      </c>
-      <c r="B23" s="10" t="str">
-        <f>+Attendance!B23</f>
-        <v>Day of Data St Louis 2026 (#1148)</v>
+      <c r="A23" s="24">
+        <v>46284</v>
+      </c>
+      <c r="B23" s="12" t="s">
+        <v>40</v>
       </c>
       <c r="C23">
         <v>0</v>
@@ -1883,20 +1922,18 @@
         <v>0</v>
       </c>
       <c r="H23" s="8">
-        <f>+Attendance!C23</f>
+        <f>+Attendance!C25</f>
         <v>0</v>
       </c>
       <c r="O23" s="21"/>
       <c r="P23" s="22"/>
     </row>
     <row r="24" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A24" s="10">
-        <f>+Attendance!A24</f>
-        <v>46319</v>
-      </c>
-      <c r="B24" s="10" t="str">
-        <f>+Attendance!B24</f>
-        <v>SQL Saturday Minnesota 2026 (#1153)</v>
+      <c r="A24" s="25">
+        <v>46298</v>
+      </c>
+      <c r="B24" s="12" t="s">
+        <v>35</v>
       </c>
       <c r="C24">
         <v>0</v>
@@ -1915,20 +1952,18 @@
         <v>0</v>
       </c>
       <c r="H24" s="8">
-        <f>+Attendance!C24</f>
+        <f>+Attendance!C26</f>
         <v>0</v>
       </c>
       <c r="O24" s="21"/>
       <c r="P24" s="22"/>
     </row>
     <row r="25" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A25" s="10">
-        <f>+Attendance!A25</f>
-        <v>46333</v>
-      </c>
-      <c r="B25" s="10" t="str">
-        <f>+Attendance!B25</f>
-        <v>Day of Data PNW 2026 (#1149)</v>
+      <c r="A25" s="25">
+        <v>46319</v>
+      </c>
+      <c r="B25" s="12" t="s">
+        <v>36</v>
       </c>
       <c r="C25">
         <v>0</v>
@@ -1947,25 +1982,69 @@
         <v>0</v>
       </c>
       <c r="H25" s="8">
-        <f>+Attendance!C25</f>
+        <f>+Attendance!C27</f>
         <v>0</v>
       </c>
       <c r="O25" s="21"/>
       <c r="P25" s="22"/>
     </row>
     <row r="26" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A26" s="10">
-        <f>+Attendance!A26</f>
-        <v>0</v>
-      </c>
-      <c r="B26" s="10">
-        <f>+Attendance!B26</f>
+      <c r="A26" s="25">
+        <v>46319</v>
+      </c>
+      <c r="B26" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="C26">
+        <v>0</v>
+      </c>
+      <c r="D26">
+        <v>0</v>
+      </c>
+      <c r="E26">
+        <v>0</v>
+      </c>
+      <c r="F26">
+        <v>0</v>
+      </c>
+      <c r="G26" s="8">
+        <f t="shared" ref="G26:G27" si="5">+H26-SUM(C26:F26)</f>
+        <v>0</v>
+      </c>
+      <c r="H26" s="8">
+        <f>+Attendance!C28</f>
         <v>0</v>
       </c>
       <c r="O26" s="21"/>
       <c r="P26" s="22"/>
     </row>
     <row r="27" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A27" s="25">
+        <v>46333</v>
+      </c>
+      <c r="B27" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="C27">
+        <v>0</v>
+      </c>
+      <c r="D27">
+        <v>0</v>
+      </c>
+      <c r="E27">
+        <v>0</v>
+      </c>
+      <c r="F27">
+        <v>0</v>
+      </c>
+      <c r="G27" s="8">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="H27" s="8">
+        <f>+Attendance!C29</f>
+        <v>0</v>
+      </c>
       <c r="O27" s="21"/>
       <c r="P27" s="22"/>
     </row>
@@ -1981,7 +2060,16 @@
   <mergeCells count="1">
     <mergeCell ref="P6:P7"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="B22" r:id="rId1" display="https://sqlsaturday.com/2026-09-19-sqlsaturday1152/" xr:uid="{0D6A567B-FCB7-44A2-A51E-648C719A8354}"/>
+    <hyperlink ref="B24" r:id="rId2" display="https://sqlsaturday.com/2026-10-03-sqlsaturday1150/" xr:uid="{D31F3CEB-8FBE-4CA1-97BB-2A40A92A8401}"/>
+    <hyperlink ref="B25" r:id="rId3" display="https://sqlsaturday.com/2026-10-24-sqlsaturday1148/" xr:uid="{96299D66-5563-46A3-B76A-F680ABDD2206}"/>
+    <hyperlink ref="B26" r:id="rId4" display="https://sqlsaturday.com/2026-10-24-sqlsaturday1153/" xr:uid="{4FAC5D40-7DBE-4A53-AFF9-C92E65F31759}"/>
+    <hyperlink ref="B27" r:id="rId5" display="https://sqlsaturday.com/2026-11-07-sqlsaturday1149/" xr:uid="{45E94655-95AF-4485-A5A2-4A3DD7455E27}"/>
+    <hyperlink ref="B21" r:id="rId6" display="https://sqlsaturday.com/2026-09-12-sqlsaturday1164/" xr:uid="{5E7F8464-7EFE-4379-AF7A-413F4F14ABD5}"/>
+    <hyperlink ref="B23" r:id="rId7" display="https://sqlsaturday.com/2026-09-19-sqlsaturday1156/" xr:uid="{840B9723-899E-4E77-BBFA-21BF1FA89943}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId8"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
attendance and other updtes (#1422)
Co-authored-by: way0utwest <admin@sqlsaturday.com>
</commit_message>
<xml_diff>
--- a/assets/misc/2026/2026_Attendance.xlsx
+++ b/assets/misc/2026/2026_Attendance.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Documents\git\sqlsatwebsite\assets\misc\2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2EAE2CA-1540-470A-AC36-A41872D3AC98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{054AC06E-9201-4BD6-9BC0-C5AEA7B3676E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15990" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2190" yWindow="45" windowWidth="22995" windowHeight="15165" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Attendance" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="41">
   <si>
     <t>Date</t>
   </si>
@@ -151,6 +151,12 @@
   </si>
   <si>
     <t>Day of Data PNW 2026 (#1149)</t>
+  </si>
+  <si>
+    <t>Day of Data Detroit 2026 (#1164)</t>
+  </si>
+  <si>
+    <t>Day of Data Vitória 2026 (#1156)</t>
   </si>
 </sst>
 </file>
@@ -239,7 +245,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -298,6 +304,8 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1"/>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Comma" xfId="2" builtinId="3"/>
@@ -605,7 +613,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:I33"/>
+  <dimension ref="A1:I35"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.7109375" style="10" bestFit="1" customWidth="1"/>
@@ -659,7 +667,7 @@
         <v>108</v>
       </c>
       <c r="E2" s="7">
-        <f t="shared" ref="E2:E26" si="0">IF(C2=0,0,+(C2-D2)/C2)</f>
+        <f t="shared" ref="E2:E28" si="0">IF(C2=0,0,+(C2-D2)/C2)</f>
         <v>0.63758389261744963</v>
       </c>
     </row>
@@ -962,14 +970,14 @@
         <v>33</v>
       </c>
       <c r="C19" s="6">
-        <v>0</v>
+        <v>128</v>
       </c>
       <c r="D19" s="6">
-        <v>0</v>
+        <v>116</v>
       </c>
       <c r="E19" s="7">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>9.375E-2</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -991,47 +999,47 @@
       </c>
     </row>
     <row r="21" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="10">
+      <c r="A21" s="5">
+        <v>46277</v>
+      </c>
+      <c r="B21" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="C21" s="6">
+        <v>0</v>
+      </c>
+      <c r="D21" s="6">
+        <v>0</v>
+      </c>
+      <c r="E21" s="7">
+        <f t="shared" ref="E21" si="1">IF(C21=0,0,+(C21-D21)/C21)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="10">
         <v>46284</v>
       </c>
-      <c r="B21" s="12" t="s">
+      <c r="B22" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="C21" s="6">
-        <v>0</v>
-      </c>
-      <c r="D21" s="6">
-        <v>0</v>
-      </c>
-      <c r="E21" s="7">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="5">
-        <v>46298</v>
-      </c>
-      <c r="B22" s="12" t="s">
-        <v>35</v>
-      </c>
       <c r="C22" s="6">
-        <v>0</v>
+        <v>140</v>
       </c>
       <c r="D22" s="6">
-        <v>0</v>
+        <v>65</v>
       </c>
       <c r="E22" s="7">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.5357142857142857</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="5">
-        <v>46319</v>
+      <c r="A23" s="10">
+        <v>46284</v>
       </c>
       <c r="B23" s="12" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C23" s="6">
         <v>0</v>
@@ -1040,16 +1048,16 @@
         <v>0</v>
       </c>
       <c r="E23" s="7">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="E23" si="2">IF(C23=0,0,+(C23-D23)/C23)</f>
         <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="5">
-        <v>46319</v>
+        <v>46298</v>
       </c>
       <c r="B24" s="12" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C24" s="6">
         <v>0</v>
@@ -1064,48 +1072,74 @@
     </row>
     <row r="25" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="5">
+        <v>46319</v>
+      </c>
+      <c r="B25" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="C25" s="6">
+        <v>0</v>
+      </c>
+      <c r="D25" s="6">
+        <v>0</v>
+      </c>
+      <c r="E25" s="7">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="5">
+        <v>46319</v>
+      </c>
+      <c r="B26" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="C26" s="6">
+        <v>0</v>
+      </c>
+      <c r="D26" s="6">
+        <v>0</v>
+      </c>
+      <c r="E26" s="7">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="5">
         <v>46333</v>
       </c>
-      <c r="B25" s="12" t="s">
+      <c r="B27" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="C25" s="6">
-        <v>0</v>
-      </c>
-      <c r="D25" s="6">
-        <v>0</v>
-      </c>
-      <c r="E25" s="7">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="5"/>
-      <c r="B26" s="12"/>
-      <c r="E26" s="7">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="5"/>
-      <c r="B27" s="12"/>
-      <c r="E27" s="7"/>
+      <c r="C27" s="6">
+        <v>0</v>
+      </c>
+      <c r="D27" s="6">
+        <v>0</v>
+      </c>
+      <c r="E27" s="7">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="28" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="5"/>
-      <c r="B28" s="13"/>
-      <c r="E28" s="7"/>
-    </row>
-    <row r="29" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B28" s="12"/>
+      <c r="E28" s="7">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="5"/>
-      <c r="B29" s="9"/>
+      <c r="B29" s="12"/>
       <c r="E29" s="7"/>
     </row>
     <row r="30" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="5"/>
-      <c r="B30" s="9"/>
+      <c r="B30" s="13"/>
       <c r="E30" s="7"/>
     </row>
     <row r="31" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1123,9 +1157,19 @@
       <c r="B33" s="9"/>
       <c r="E33" s="7"/>
     </row>
+    <row r="34" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="5"/>
+      <c r="B34" s="9"/>
+      <c r="E34" s="7"/>
+    </row>
+    <row r="35" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="5"/>
+      <c r="B35" s="9"/>
+      <c r="E35" s="7"/>
+    </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I34">
-    <sortCondition ref="A2:A34"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I36">
+    <sortCondition ref="A2:A36"/>
   </sortState>
   <hyperlinks>
     <hyperlink ref="B2" r:id="rId1" display="https://sqlsaturday.com/2026-01-17-sqlsaturday1138/" xr:uid="{82BDF17B-780C-46C4-BDF3-6B50D2949365}"/>
@@ -1147,14 +1191,16 @@
     <hyperlink ref="B17" r:id="rId17" display="https://sqlsaturday.com/2026-06-27-sqlsaturday1154/" xr:uid="{4E193433-7FEF-42F0-9BE1-2E1B4F56DC45}"/>
     <hyperlink ref="B18" r:id="rId18" display="https://sqlsaturday.com/2026-07-18-sqlsaturday1141/" xr:uid="{B4310BB2-BE85-4D94-9531-7F04382A3C59}"/>
     <hyperlink ref="B19" r:id="rId19" display="https://sqlsaturday.com/2026-08-08-sqlsaturday1144/" xr:uid="{49013F68-7251-4303-A8A8-19F4C344B133}"/>
-    <hyperlink ref="B21" r:id="rId20" display="https://sqlsaturday.com/2026-09-19-sqlsaturday1152/" xr:uid="{1C24212F-ACFE-4FD3-A6CF-8E691EEA9C75}"/>
-    <hyperlink ref="B22" r:id="rId21" display="https://sqlsaturday.com/2026-10-03-sqlsaturday1150/" xr:uid="{80072270-983F-4E6A-AFAE-3FC24DE448B3}"/>
-    <hyperlink ref="B23" r:id="rId22" display="https://sqlsaturday.com/2026-10-24-sqlsaturday1148/" xr:uid="{111A5B01-58C6-46AB-81AC-567A7B3C8861}"/>
-    <hyperlink ref="B24" r:id="rId23" display="https://sqlsaturday.com/2026-10-24-sqlsaturday1153/" xr:uid="{29A122E2-6150-4028-BEF4-E884CED9AA91}"/>
-    <hyperlink ref="B25" r:id="rId24" display="https://sqlsaturday.com/2026-11-07-sqlsaturday1149/" xr:uid="{1C87B471-8BB8-47E8-8A2F-FEB250EAF056}"/>
+    <hyperlink ref="B22" r:id="rId20" display="https://sqlsaturday.com/2026-09-19-sqlsaturday1152/" xr:uid="{1C24212F-ACFE-4FD3-A6CF-8E691EEA9C75}"/>
+    <hyperlink ref="B24" r:id="rId21" display="https://sqlsaturday.com/2026-10-03-sqlsaturday1150/" xr:uid="{80072270-983F-4E6A-AFAE-3FC24DE448B3}"/>
+    <hyperlink ref="B25" r:id="rId22" display="https://sqlsaturday.com/2026-10-24-sqlsaturday1148/" xr:uid="{111A5B01-58C6-46AB-81AC-567A7B3C8861}"/>
+    <hyperlink ref="B26" r:id="rId23" display="https://sqlsaturday.com/2026-10-24-sqlsaturday1153/" xr:uid="{29A122E2-6150-4028-BEF4-E884CED9AA91}"/>
+    <hyperlink ref="B27" r:id="rId24" display="https://sqlsaturday.com/2026-11-07-sqlsaturday1149/" xr:uid="{1C87B471-8BB8-47E8-8A2F-FEB250EAF056}"/>
+    <hyperlink ref="B21" r:id="rId25" display="https://sqlsaturday.com/2026-09-12-sqlsaturday1164/" xr:uid="{C31C9E88-D474-46E9-9D7F-515DB0D1C4FD}"/>
+    <hyperlink ref="B23" r:id="rId26" display="https://sqlsaturday.com/2026-09-19-sqlsaturday1156/" xr:uid="{D29C5250-03B6-490D-8B76-A7A1B304D760}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId25"/>
+  <pageSetup orientation="portrait" r:id="rId27"/>
 </worksheet>
 </file>
 
@@ -1196,7 +1242,7 @@
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A2" s="10">
+      <c r="A2" s="24">
         <f>+Attendance!A2</f>
         <v>46039</v>
       </c>
@@ -1226,7 +1272,7 @@
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A3" s="10">
+      <c r="A3" s="24">
         <f>+Attendance!A3</f>
         <v>46102</v>
       </c>
@@ -1256,7 +1302,7 @@
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A4" s="10">
+      <c r="A4" s="24">
         <f>+Attendance!A4</f>
         <v>46109</v>
       </c>
@@ -1286,7 +1332,7 @@
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A5" s="10">
+      <c r="A5" s="24">
         <f>+Attendance!A5</f>
         <v>46123</v>
       </c>
@@ -1316,7 +1362,7 @@
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A6" s="10">
+      <c r="A6" s="24">
         <f>+Attendance!A6</f>
         <v>46123</v>
       </c>
@@ -1348,7 +1394,7 @@
       <c r="P6" s="23"/>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A7" s="10">
+      <c r="A7" s="24">
         <f>+Attendance!A7</f>
         <v>46130</v>
       </c>
@@ -1381,7 +1427,7 @@
       <c r="P7" s="23"/>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A8" s="10">
+      <c r="A8" s="24">
         <f>+Attendance!A8</f>
         <v>46137</v>
       </c>
@@ -1413,7 +1459,7 @@
       <c r="P8" s="22"/>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A9" s="10">
+      <c r="A9" s="24">
         <f>+Attendance!A9</f>
         <v>46137</v>
       </c>
@@ -1445,7 +1491,7 @@
       <c r="P9" s="22"/>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A10" s="10">
+      <c r="A10" s="24">
         <f>+Attendance!A10</f>
         <v>46144</v>
       </c>
@@ -1477,7 +1523,7 @@
       <c r="P10" s="22"/>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A11" s="10">
+      <c r="A11" s="24">
         <f>+Attendance!A11</f>
         <v>46158</v>
       </c>
@@ -1509,7 +1555,7 @@
       <c r="P11" s="22"/>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A12" s="10">
+      <c r="A12" s="24">
         <f>+Attendance!A12</f>
         <v>46256</v>
       </c>
@@ -1541,7 +1587,7 @@
       <c r="P12" s="22"/>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A13" s="10">
+      <c r="A13" s="24">
         <f>+Attendance!A13</f>
         <v>46165</v>
       </c>
@@ -1573,7 +1619,7 @@
       <c r="P13" s="22"/>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A14" s="10">
+      <c r="A14" s="24">
         <f>+Attendance!A14</f>
         <v>46172</v>
       </c>
@@ -1604,7 +1650,7 @@
       <c r="P14" s="22"/>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A15" s="10">
+      <c r="A15" s="24">
         <f>+Attendance!A15</f>
         <v>46186</v>
       </c>
@@ -1635,7 +1681,7 @@
       <c r="P15" s="22"/>
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A16" s="10">
+      <c r="A16" s="24">
         <f>+Attendance!A16</f>
         <v>46200</v>
       </c>
@@ -1666,7 +1712,7 @@
       <c r="P16" s="22"/>
     </row>
     <row r="17" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A17" s="10">
+      <c r="A17" s="24">
         <f>+Attendance!A17</f>
         <v>46200</v>
       </c>
@@ -1698,7 +1744,7 @@
       <c r="P17" s="22"/>
     </row>
     <row r="18" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A18" s="10">
+      <c r="A18" s="24">
         <f>+Attendance!A18</f>
         <v>46221</v>
       </c>
@@ -1730,7 +1776,7 @@
       <c r="P18" s="22"/>
     </row>
     <row r="19" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A19" s="10">
+      <c r="A19" s="24">
         <f>+Attendance!A19</f>
         <v>46242</v>
       </c>
@@ -1742,27 +1788,26 @@
         <v>0</v>
       </c>
       <c r="D19">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="E19">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F19">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="G19" s="8">
-        <f t="shared" si="3"/>
-        <v>0</v>
+        <v>61</v>
       </c>
       <c r="H19" s="8">
         <f>+Attendance!C19</f>
-        <v>0</v>
+        <v>128</v>
       </c>
       <c r="O19" s="21"/>
       <c r="P19" s="22"/>
     </row>
     <row r="20" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A20" s="10">
+      <c r="A20" s="24">
         <f>+Attendance!A20</f>
         <v>46256</v>
       </c>
@@ -1794,13 +1839,11 @@
       <c r="P20" s="22"/>
     </row>
     <row r="21" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A21" s="10">
-        <f>+Attendance!A21</f>
-        <v>46284</v>
-      </c>
-      <c r="B21" s="10" t="str">
-        <f>+Attendance!B21</f>
-        <v>Salt Lake City Day of Data 2026 (#1152)</v>
+      <c r="A21" s="25">
+        <v>46277</v>
+      </c>
+      <c r="B21" s="12" t="s">
+        <v>39</v>
       </c>
       <c r="C21">
         <v>0</v>
@@ -1816,23 +1859,21 @@
       </c>
       <c r="G21" s="8">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>140</v>
       </c>
       <c r="H21" s="8">
-        <f>+Attendance!C21</f>
-        <v>0</v>
+        <f>+Attendance!C22</f>
+        <v>140</v>
       </c>
       <c r="O21" s="21"/>
       <c r="P21" s="22"/>
     </row>
     <row r="22" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A22" s="10">
-        <f>+Attendance!A22</f>
-        <v>46298</v>
-      </c>
-      <c r="B22" s="10" t="str">
-        <f>+Attendance!B22</f>
-        <v>Boston Data and AI Saturday 2026 (#1150)</v>
+      <c r="A22" s="24">
+        <v>46284</v>
+      </c>
+      <c r="B22" s="12" t="s">
+        <v>34</v>
       </c>
       <c r="C22">
         <v>0</v>
@@ -1851,20 +1892,18 @@
         <v>0</v>
       </c>
       <c r="H22" s="8">
-        <f>+Attendance!C22</f>
+        <f>+Attendance!C24</f>
         <v>0</v>
       </c>
       <c r="O22" s="21"/>
       <c r="P22" s="22"/>
     </row>
     <row r="23" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A23" s="10">
-        <f>+Attendance!A23</f>
-        <v>46319</v>
-      </c>
-      <c r="B23" s="10" t="str">
-        <f>+Attendance!B23</f>
-        <v>Day of Data St Louis 2026 (#1148)</v>
+      <c r="A23" s="24">
+        <v>46284</v>
+      </c>
+      <c r="B23" s="12" t="s">
+        <v>40</v>
       </c>
       <c r="C23">
         <v>0</v>
@@ -1883,20 +1922,18 @@
         <v>0</v>
       </c>
       <c r="H23" s="8">
-        <f>+Attendance!C23</f>
+        <f>+Attendance!C25</f>
         <v>0</v>
       </c>
       <c r="O23" s="21"/>
       <c r="P23" s="22"/>
     </row>
     <row r="24" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A24" s="10">
-        <f>+Attendance!A24</f>
-        <v>46319</v>
-      </c>
-      <c r="B24" s="10" t="str">
-        <f>+Attendance!B24</f>
-        <v>SQL Saturday Minnesota 2026 (#1153)</v>
+      <c r="A24" s="25">
+        <v>46298</v>
+      </c>
+      <c r="B24" s="12" t="s">
+        <v>35</v>
       </c>
       <c r="C24">
         <v>0</v>
@@ -1915,20 +1952,18 @@
         <v>0</v>
       </c>
       <c r="H24" s="8">
-        <f>+Attendance!C24</f>
+        <f>+Attendance!C26</f>
         <v>0</v>
       </c>
       <c r="O24" s="21"/>
       <c r="P24" s="22"/>
     </row>
     <row r="25" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A25" s="10">
-        <f>+Attendance!A25</f>
-        <v>46333</v>
-      </c>
-      <c r="B25" s="10" t="str">
-        <f>+Attendance!B25</f>
-        <v>Day of Data PNW 2026 (#1149)</v>
+      <c r="A25" s="25">
+        <v>46319</v>
+      </c>
+      <c r="B25" s="12" t="s">
+        <v>36</v>
       </c>
       <c r="C25">
         <v>0</v>
@@ -1947,25 +1982,69 @@
         <v>0</v>
       </c>
       <c r="H25" s="8">
-        <f>+Attendance!C25</f>
+        <f>+Attendance!C27</f>
         <v>0</v>
       </c>
       <c r="O25" s="21"/>
       <c r="P25" s="22"/>
     </row>
     <row r="26" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A26" s="10">
-        <f>+Attendance!A26</f>
-        <v>0</v>
-      </c>
-      <c r="B26" s="10">
-        <f>+Attendance!B26</f>
+      <c r="A26" s="25">
+        <v>46319</v>
+      </c>
+      <c r="B26" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="C26">
+        <v>0</v>
+      </c>
+      <c r="D26">
+        <v>0</v>
+      </c>
+      <c r="E26">
+        <v>0</v>
+      </c>
+      <c r="F26">
+        <v>0</v>
+      </c>
+      <c r="G26" s="8">
+        <f t="shared" ref="G26:G27" si="5">+H26-SUM(C26:F26)</f>
+        <v>0</v>
+      </c>
+      <c r="H26" s="8">
+        <f>+Attendance!C28</f>
         <v>0</v>
       </c>
       <c r="O26" s="21"/>
       <c r="P26" s="22"/>
     </row>
     <row r="27" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A27" s="25">
+        <v>46333</v>
+      </c>
+      <c r="B27" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="C27">
+        <v>0</v>
+      </c>
+      <c r="D27">
+        <v>0</v>
+      </c>
+      <c r="E27">
+        <v>0</v>
+      </c>
+      <c r="F27">
+        <v>0</v>
+      </c>
+      <c r="G27" s="8">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="H27" s="8">
+        <f>+Attendance!C29</f>
+        <v>0</v>
+      </c>
       <c r="O27" s="21"/>
       <c r="P27" s="22"/>
     </row>
@@ -1981,7 +2060,16 @@
   <mergeCells count="1">
     <mergeCell ref="P6:P7"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="B22" r:id="rId1" display="https://sqlsaturday.com/2026-09-19-sqlsaturday1152/" xr:uid="{0D6A567B-FCB7-44A2-A51E-648C719A8354}"/>
+    <hyperlink ref="B24" r:id="rId2" display="https://sqlsaturday.com/2026-10-03-sqlsaturday1150/" xr:uid="{D31F3CEB-8FBE-4CA1-97BB-2A40A92A8401}"/>
+    <hyperlink ref="B25" r:id="rId3" display="https://sqlsaturday.com/2026-10-24-sqlsaturday1148/" xr:uid="{96299D66-5563-46A3-B76A-F680ABDD2206}"/>
+    <hyperlink ref="B26" r:id="rId4" display="https://sqlsaturday.com/2026-10-24-sqlsaturday1153/" xr:uid="{4FAC5D40-7DBE-4A53-AFF9-C92E65F31759}"/>
+    <hyperlink ref="B27" r:id="rId5" display="https://sqlsaturday.com/2026-11-07-sqlsaturday1149/" xr:uid="{45E94655-95AF-4485-A5A2-4A3DD7455E27}"/>
+    <hyperlink ref="B21" r:id="rId6" display="https://sqlsaturday.com/2026-09-12-sqlsaturday1164/" xr:uid="{5E7F8464-7EFE-4379-AF7A-413F4F14ABD5}"/>
+    <hyperlink ref="B23" r:id="rId7" display="https://sqlsaturday.com/2026-09-19-sqlsaturday1156/" xr:uid="{840B9723-899E-4E77-BBFA-21BF1FA89943}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId8"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
updates from detroit and winnipeg
</commit_message>
<xml_diff>
--- a/assets/misc/2026/2026_Attendance.xlsx
+++ b/assets/misc/2026/2026_Attendance.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Documents\git\sqlsatwebsite\assets\misc\2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{054AC06E-9201-4BD6-9BC0-C5AEA7B3676E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DD2463E-D8D7-4C9F-BCC8-D066D73F5C3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2190" yWindow="45" windowWidth="22995" windowHeight="15165" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1005" yWindow="165" windowWidth="25260" windowHeight="15210" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Attendance" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="42">
   <si>
     <t>Date</t>
   </si>
@@ -157,6 +157,9 @@
   </si>
   <si>
     <t>Day of Data Vitória 2026 (#1156)</t>
+  </si>
+  <si>
+    <t>Day of Data Winnipeg 2026 (#1159)</t>
   </si>
 </sst>
 </file>
@@ -245,7 +248,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -301,11 +304,10 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1"/>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Comma" xfId="2" builtinId="3"/>
@@ -613,7 +615,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:I35"/>
+  <dimension ref="A1:I36"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.7109375" style="10" bestFit="1" customWidth="1"/>
@@ -667,7 +669,7 @@
         <v>108</v>
       </c>
       <c r="E2" s="7">
-        <f t="shared" ref="E2:E28" si="0">IF(C2=0,0,+(C2-D2)/C2)</f>
+        <f t="shared" ref="E2:E29" si="0">IF(C2=0,0,+(C2-D2)/C2)</f>
         <v>0.63758389261744963</v>
       </c>
     </row>
@@ -1006,14 +1008,14 @@
         <v>39</v>
       </c>
       <c r="C21" s="6">
-        <v>0</v>
+        <v>96</v>
       </c>
       <c r="D21" s="6">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="E21" s="7">
         <f t="shared" ref="E21" si="1">IF(C21=0,0,+(C21-D21)/C21)</f>
-        <v>0</v>
+        <v>0.47916666666666669</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1048,34 +1050,34 @@
         <v>0</v>
       </c>
       <c r="E23" s="7">
-        <f t="shared" ref="E23" si="2">IF(C23=0,0,+(C23-D23)/C23)</f>
+        <f t="shared" ref="E23:E24" si="2">IF(C23=0,0,+(C23-D23)/C23)</f>
         <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="5">
-        <v>46298</v>
+      <c r="A24" s="10">
+        <v>46284</v>
       </c>
       <c r="B24" s="12" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="C24" s="6">
-        <v>0</v>
+        <v>363</v>
       </c>
       <c r="D24" s="6">
-        <v>0</v>
+        <v>163</v>
       </c>
       <c r="E24" s="7">
-        <f t="shared" si="0"/>
-        <v>0</v>
+        <f t="shared" si="2"/>
+        <v>0.55096418732782371</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="5">
-        <v>46319</v>
+        <v>46298</v>
       </c>
       <c r="B25" s="12" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C25" s="6">
         <v>0</v>
@@ -1093,7 +1095,7 @@
         <v>46319</v>
       </c>
       <c r="B26" s="12" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C26" s="6">
         <v>0</v>
@@ -1108,43 +1110,56 @@
     </row>
     <row r="27" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="5">
+        <v>46319</v>
+      </c>
+      <c r="B27" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="C27" s="6">
+        <v>0</v>
+      </c>
+      <c r="D27" s="6">
+        <v>0</v>
+      </c>
+      <c r="E27" s="7">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="5">
         <v>46333</v>
       </c>
-      <c r="B27" s="12" t="s">
+      <c r="B28" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="C27" s="6">
-        <v>0</v>
-      </c>
-      <c r="D27" s="6">
-        <v>0</v>
-      </c>
-      <c r="E27" s="7">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="5"/>
-      <c r="B28" s="12"/>
+      <c r="C28" s="6">
+        <v>0</v>
+      </c>
+      <c r="D28" s="6">
+        <v>0</v>
+      </c>
       <c r="E28" s="7">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="5"/>
       <c r="B29" s="12"/>
-      <c r="E29" s="7"/>
-    </row>
-    <row r="30" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E29" s="7">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="5"/>
-      <c r="B30" s="13"/>
+      <c r="B30" s="12"/>
       <c r="E30" s="7"/>
     </row>
     <row r="31" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="5"/>
-      <c r="B31" s="9"/>
+      <c r="B31" s="13"/>
       <c r="E31" s="7"/>
     </row>
     <row r="32" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1167,9 +1182,14 @@
       <c r="B35" s="9"/>
       <c r="E35" s="7"/>
     </row>
+    <row r="36" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="5"/>
+      <c r="B36" s="9"/>
+      <c r="E36" s="7"/>
+    </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I36">
-    <sortCondition ref="A2:A36"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I37">
+    <sortCondition ref="A2:A37"/>
   </sortState>
   <hyperlinks>
     <hyperlink ref="B2" r:id="rId1" display="https://sqlsaturday.com/2026-01-17-sqlsaturday1138/" xr:uid="{82BDF17B-780C-46C4-BDF3-6B50D2949365}"/>
@@ -1192,21 +1212,22 @@
     <hyperlink ref="B18" r:id="rId18" display="https://sqlsaturday.com/2026-07-18-sqlsaturday1141/" xr:uid="{B4310BB2-BE85-4D94-9531-7F04382A3C59}"/>
     <hyperlink ref="B19" r:id="rId19" display="https://sqlsaturday.com/2026-08-08-sqlsaturday1144/" xr:uid="{49013F68-7251-4303-A8A8-19F4C344B133}"/>
     <hyperlink ref="B22" r:id="rId20" display="https://sqlsaturday.com/2026-09-19-sqlsaturday1152/" xr:uid="{1C24212F-ACFE-4FD3-A6CF-8E691EEA9C75}"/>
-    <hyperlink ref="B24" r:id="rId21" display="https://sqlsaturday.com/2026-10-03-sqlsaturday1150/" xr:uid="{80072270-983F-4E6A-AFAE-3FC24DE448B3}"/>
-    <hyperlink ref="B25" r:id="rId22" display="https://sqlsaturday.com/2026-10-24-sqlsaturday1148/" xr:uid="{111A5B01-58C6-46AB-81AC-567A7B3C8861}"/>
-    <hyperlink ref="B26" r:id="rId23" display="https://sqlsaturday.com/2026-10-24-sqlsaturday1153/" xr:uid="{29A122E2-6150-4028-BEF4-E884CED9AA91}"/>
-    <hyperlink ref="B27" r:id="rId24" display="https://sqlsaturday.com/2026-11-07-sqlsaturday1149/" xr:uid="{1C87B471-8BB8-47E8-8A2F-FEB250EAF056}"/>
+    <hyperlink ref="B25" r:id="rId21" display="https://sqlsaturday.com/2026-10-03-sqlsaturday1150/" xr:uid="{80072270-983F-4E6A-AFAE-3FC24DE448B3}"/>
+    <hyperlink ref="B26" r:id="rId22" display="https://sqlsaturday.com/2026-10-24-sqlsaturday1148/" xr:uid="{111A5B01-58C6-46AB-81AC-567A7B3C8861}"/>
+    <hyperlink ref="B27" r:id="rId23" display="https://sqlsaturday.com/2026-10-24-sqlsaturday1153/" xr:uid="{29A122E2-6150-4028-BEF4-E884CED9AA91}"/>
+    <hyperlink ref="B28" r:id="rId24" display="https://sqlsaturday.com/2026-11-07-sqlsaturday1149/" xr:uid="{1C87B471-8BB8-47E8-8A2F-FEB250EAF056}"/>
     <hyperlink ref="B21" r:id="rId25" display="https://sqlsaturday.com/2026-09-12-sqlsaturday1164/" xr:uid="{C31C9E88-D474-46E9-9D7F-515DB0D1C4FD}"/>
     <hyperlink ref="B23" r:id="rId26" display="https://sqlsaturday.com/2026-09-19-sqlsaturday1156/" xr:uid="{D29C5250-03B6-490D-8B76-A7A1B304D760}"/>
+    <hyperlink ref="B24" r:id="rId27" display="https://sqlsaturday.com/2026-09-19-sqlsaturday1159/" xr:uid="{120DA250-32FF-4D5E-BAA0-AE998F27E101}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId27"/>
+  <pageSetup orientation="portrait" r:id="rId28"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C9FAEBE-70DD-4114-ACD9-DE4988A37B44}">
-  <dimension ref="A1:P29"/>
+  <dimension ref="A1:P30"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -1242,7 +1263,7 @@
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A2" s="24">
+      <c r="A2" s="10">
         <f>+Attendance!A2</f>
         <v>46039</v>
       </c>
@@ -1272,7 +1293,7 @@
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A3" s="24">
+      <c r="A3" s="10">
         <f>+Attendance!A3</f>
         <v>46102</v>
       </c>
@@ -1302,7 +1323,7 @@
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A4" s="24">
+      <c r="A4" s="10">
         <f>+Attendance!A4</f>
         <v>46109</v>
       </c>
@@ -1332,7 +1353,7 @@
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A5" s="24">
+      <c r="A5" s="10">
         <f>+Attendance!A5</f>
         <v>46123</v>
       </c>
@@ -1362,7 +1383,7 @@
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A6" s="24">
+      <c r="A6" s="10">
         <f>+Attendance!A6</f>
         <v>46123</v>
       </c>
@@ -1391,10 +1412,10 @@
         <v>167</v>
       </c>
       <c r="O6" s="20"/>
-      <c r="P6" s="23"/>
+      <c r="P6" s="24"/>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A7" s="24">
+      <c r="A7" s="10">
         <f>+Attendance!A7</f>
         <v>46130</v>
       </c>
@@ -1424,10 +1445,10 @@
         <v>134</v>
       </c>
       <c r="O7" s="21"/>
-      <c r="P7" s="23"/>
+      <c r="P7" s="24"/>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A8" s="24">
+      <c r="A8" s="10">
         <f>+Attendance!A8</f>
         <v>46137</v>
       </c>
@@ -1459,7 +1480,7 @@
       <c r="P8" s="22"/>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A9" s="24">
+      <c r="A9" s="10">
         <f>+Attendance!A9</f>
         <v>46137</v>
       </c>
@@ -1491,7 +1512,7 @@
       <c r="P9" s="22"/>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A10" s="24">
+      <c r="A10" s="10">
         <f>+Attendance!A10</f>
         <v>46144</v>
       </c>
@@ -1523,7 +1544,7 @@
       <c r="P10" s="22"/>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A11" s="24">
+      <c r="A11" s="10">
         <f>+Attendance!A11</f>
         <v>46158</v>
       </c>
@@ -1555,7 +1576,7 @@
       <c r="P11" s="22"/>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A12" s="24">
+      <c r="A12" s="10">
         <f>+Attendance!A12</f>
         <v>46256</v>
       </c>
@@ -1587,7 +1608,7 @@
       <c r="P12" s="22"/>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A13" s="24">
+      <c r="A13" s="10">
         <f>+Attendance!A13</f>
         <v>46165</v>
       </c>
@@ -1608,7 +1629,7 @@
         <v>0</v>
       </c>
       <c r="G13" s="8">
-        <f t="shared" ref="G13:G24" si="3">+H13-SUM(C13:F13)</f>
+        <f t="shared" ref="G13:G25" si="3">+H13-SUM(C13:F13)</f>
         <v>178</v>
       </c>
       <c r="H13" s="8">
@@ -1619,7 +1640,7 @@
       <c r="P13" s="22"/>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A14" s="24">
+      <c r="A14" s="10">
         <f>+Attendance!A14</f>
         <v>46172</v>
       </c>
@@ -1650,7 +1671,7 @@
       <c r="P14" s="22"/>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A15" s="24">
+      <c r="A15" s="10">
         <f>+Attendance!A15</f>
         <v>46186</v>
       </c>
@@ -1681,7 +1702,7 @@
       <c r="P15" s="22"/>
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A16" s="24">
+      <c r="A16" s="10">
         <f>+Attendance!A16</f>
         <v>46200</v>
       </c>
@@ -1712,7 +1733,7 @@
       <c r="P16" s="22"/>
     </row>
     <row r="17" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A17" s="24">
+      <c r="A17" s="10">
         <f>+Attendance!A17</f>
         <v>46200</v>
       </c>
@@ -1744,7 +1765,7 @@
       <c r="P17" s="22"/>
     </row>
     <row r="18" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A18" s="24">
+      <c r="A18" s="10">
         <f>+Attendance!A18</f>
         <v>46221</v>
       </c>
@@ -1776,7 +1797,7 @@
       <c r="P18" s="22"/>
     </row>
     <row r="19" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A19" s="24">
+      <c r="A19" s="10">
         <f>+Attendance!A19</f>
         <v>46242</v>
       </c>
@@ -1807,7 +1828,7 @@
       <c r="P19" s="22"/>
     </row>
     <row r="20" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A20" s="24">
+      <c r="A20" s="10">
         <f>+Attendance!A20</f>
         <v>46256</v>
       </c>
@@ -1839,67 +1860,67 @@
       <c r="P20" s="22"/>
     </row>
     <row r="21" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A21" s="25">
+      <c r="A21" s="23">
         <v>46277</v>
       </c>
       <c r="B21" s="12" t="s">
         <v>39</v>
       </c>
       <c r="C21">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="D21">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="E21">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F21">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="G21" s="8">
         <f t="shared" si="3"/>
+        <v>54</v>
+      </c>
+      <c r="H21" s="8">
+        <f>+Attendance!C21</f>
+        <v>96</v>
+      </c>
+      <c r="O21" s="21"/>
+      <c r="P21" s="22"/>
+    </row>
+    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A22" s="10">
+        <v>46284</v>
+      </c>
+      <c r="B22" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="C22">
+        <v>0</v>
+      </c>
+      <c r="D22">
+        <v>0</v>
+      </c>
+      <c r="E22">
+        <v>0</v>
+      </c>
+      <c r="F22">
+        <v>0</v>
+      </c>
+      <c r="G22" s="8">
+        <f t="shared" si="3"/>
         <v>140</v>
       </c>
-      <c r="H21" s="8">
+      <c r="H22" s="8">
         <f>+Attendance!C22</f>
         <v>140</v>
       </c>
-      <c r="O21" s="21"/>
-      <c r="P21" s="22"/>
-    </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A22" s="24">
-        <v>46284</v>
-      </c>
-      <c r="B22" s="12" t="s">
-        <v>34</v>
-      </c>
-      <c r="C22">
-        <v>0</v>
-      </c>
-      <c r="D22">
-        <v>0</v>
-      </c>
-      <c r="E22">
-        <v>0</v>
-      </c>
-      <c r="F22">
-        <v>0</v>
-      </c>
-      <c r="G22" s="8">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="H22" s="8">
-        <f>+Attendance!C24</f>
-        <v>0</v>
-      </c>
       <c r="O22" s="21"/>
       <c r="P22" s="22"/>
     </row>
     <row r="23" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A23" s="24">
+      <c r="A23" s="10">
         <v>46284</v>
       </c>
       <c r="B23" s="12" t="s">
@@ -1922,48 +1943,48 @@
         <v>0</v>
       </c>
       <c r="H23" s="8">
-        <f>+Attendance!C25</f>
+        <f>+Attendance!C23</f>
         <v>0</v>
       </c>
       <c r="O23" s="21"/>
       <c r="P23" s="22"/>
     </row>
     <row r="24" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A24" s="25">
-        <v>46298</v>
+      <c r="A24" s="10">
+        <v>46284</v>
       </c>
       <c r="B24" s="12" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="C24">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="D24">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E24">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F24">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="G24" s="8">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>324</v>
       </c>
       <c r="H24" s="8">
-        <f>+Attendance!C26</f>
-        <v>0</v>
+        <f>+Attendance!C24</f>
+        <v>363</v>
       </c>
       <c r="O24" s="21"/>
       <c r="P24" s="22"/>
     </row>
     <row r="25" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A25" s="25">
-        <v>46319</v>
+      <c r="A25" s="23">
+        <v>46298</v>
       </c>
       <c r="B25" s="12" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C25">
         <v>0</v>
@@ -1978,22 +1999,22 @@
         <v>0</v>
       </c>
       <c r="G25" s="8">
-        <f t="shared" ref="G25" si="4">+H25-SUM(C25:F25)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="H25" s="8">
-        <f>+Attendance!C27</f>
+        <f>+Attendance!C25</f>
         <v>0</v>
       </c>
       <c r="O25" s="21"/>
       <c r="P25" s="22"/>
     </row>
     <row r="26" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A26" s="25">
+      <c r="A26" s="23">
         <v>46319</v>
       </c>
       <c r="B26" s="12" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C26">
         <v>0</v>
@@ -2008,22 +2029,22 @@
         <v>0</v>
       </c>
       <c r="G26" s="8">
-        <f t="shared" ref="G26:G27" si="5">+H26-SUM(C26:F26)</f>
+        <f t="shared" ref="G26" si="4">+H26-SUM(C26:F26)</f>
         <v>0</v>
       </c>
       <c r="H26" s="8">
-        <f>+Attendance!C28</f>
+        <f>+Attendance!C26</f>
         <v>0</v>
       </c>
       <c r="O26" s="21"/>
       <c r="P26" s="22"/>
     </row>
     <row r="27" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A27" s="25">
-        <v>46333</v>
+      <c r="A27" s="23">
+        <v>46319</v>
       </c>
       <c r="B27" s="12" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C27">
         <v>0</v>
@@ -2038,23 +2059,53 @@
         <v>0</v>
       </c>
       <c r="G27" s="8">
-        <f t="shared" si="5"/>
+        <f t="shared" ref="G27:G28" si="5">+H27-SUM(C27:F27)</f>
         <v>0</v>
       </c>
       <c r="H27" s="8">
-        <f>+Attendance!C29</f>
+        <f>+Attendance!C27</f>
         <v>0</v>
       </c>
       <c r="O27" s="21"/>
       <c r="P27" s="22"/>
     </row>
     <row r="28" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A28" s="23">
+        <v>46333</v>
+      </c>
+      <c r="B28" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="C28">
+        <v>0</v>
+      </c>
+      <c r="D28">
+        <v>0</v>
+      </c>
+      <c r="E28">
+        <v>0</v>
+      </c>
+      <c r="F28">
+        <v>0</v>
+      </c>
+      <c r="G28" s="8">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="H28" s="8">
+        <f>+Attendance!C28</f>
+        <v>0</v>
+      </c>
       <c r="O28" s="21"/>
       <c r="P28" s="22"/>
     </row>
     <row r="29" spans="1:16" x14ac:dyDescent="0.25">
       <c r="O29" s="21"/>
       <c r="P29" s="22"/>
+    </row>
+    <row r="30" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="O30" s="21"/>
+      <c r="P30" s="22"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2062,14 +2113,15 @@
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="B22" r:id="rId1" display="https://sqlsaturday.com/2026-09-19-sqlsaturday1152/" xr:uid="{0D6A567B-FCB7-44A2-A51E-648C719A8354}"/>
-    <hyperlink ref="B24" r:id="rId2" display="https://sqlsaturday.com/2026-10-03-sqlsaturday1150/" xr:uid="{D31F3CEB-8FBE-4CA1-97BB-2A40A92A8401}"/>
-    <hyperlink ref="B25" r:id="rId3" display="https://sqlsaturday.com/2026-10-24-sqlsaturday1148/" xr:uid="{96299D66-5563-46A3-B76A-F680ABDD2206}"/>
-    <hyperlink ref="B26" r:id="rId4" display="https://sqlsaturday.com/2026-10-24-sqlsaturday1153/" xr:uid="{4FAC5D40-7DBE-4A53-AFF9-C92E65F31759}"/>
-    <hyperlink ref="B27" r:id="rId5" display="https://sqlsaturday.com/2026-11-07-sqlsaturday1149/" xr:uid="{45E94655-95AF-4485-A5A2-4A3DD7455E27}"/>
+    <hyperlink ref="B25" r:id="rId2" display="https://sqlsaturday.com/2026-10-03-sqlsaturday1150/" xr:uid="{D31F3CEB-8FBE-4CA1-97BB-2A40A92A8401}"/>
+    <hyperlink ref="B26" r:id="rId3" display="https://sqlsaturday.com/2026-10-24-sqlsaturday1148/" xr:uid="{96299D66-5563-46A3-B76A-F680ABDD2206}"/>
+    <hyperlink ref="B27" r:id="rId4" display="https://sqlsaturday.com/2026-10-24-sqlsaturday1153/" xr:uid="{4FAC5D40-7DBE-4A53-AFF9-C92E65F31759}"/>
+    <hyperlink ref="B28" r:id="rId5" display="https://sqlsaturday.com/2026-11-07-sqlsaturday1149/" xr:uid="{45E94655-95AF-4485-A5A2-4A3DD7455E27}"/>
     <hyperlink ref="B21" r:id="rId6" display="https://sqlsaturday.com/2026-09-12-sqlsaturday1164/" xr:uid="{5E7F8464-7EFE-4379-AF7A-413F4F14ABD5}"/>
     <hyperlink ref="B23" r:id="rId7" display="https://sqlsaturday.com/2026-09-19-sqlsaturday1156/" xr:uid="{840B9723-899E-4E77-BBFA-21BF1FA89943}"/>
+    <hyperlink ref="B24" r:id="rId8" display="https://sqlsaturday.com/2026-09-19-sqlsaturday1159/" xr:uid="{0795C785-E600-4CBB-BC80-E9889F632DF8}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId8"/>
+  <pageSetup orientation="portrait" r:id="rId9"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
updates from detroit and winnipeg (#1429)
Co-authored-by: way0utwest <admin@sqlsaturday.com>
</commit_message>
<xml_diff>
--- a/assets/misc/2026/2026_Attendance.xlsx
+++ b/assets/misc/2026/2026_Attendance.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Documents\git\sqlsatwebsite\assets\misc\2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{054AC06E-9201-4BD6-9BC0-C5AEA7B3676E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DD2463E-D8D7-4C9F-BCC8-D066D73F5C3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2190" yWindow="45" windowWidth="22995" windowHeight="15165" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1005" yWindow="165" windowWidth="25260" windowHeight="15210" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Attendance" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="42">
   <si>
     <t>Date</t>
   </si>
@@ -157,6 +157,9 @@
   </si>
   <si>
     <t>Day of Data Vitória 2026 (#1156)</t>
+  </si>
+  <si>
+    <t>Day of Data Winnipeg 2026 (#1159)</t>
   </si>
 </sst>
 </file>
@@ -245,7 +248,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -301,11 +304,10 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1"/>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Comma" xfId="2" builtinId="3"/>
@@ -613,7 +615,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:I35"/>
+  <dimension ref="A1:I36"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.7109375" style="10" bestFit="1" customWidth="1"/>
@@ -667,7 +669,7 @@
         <v>108</v>
       </c>
       <c r="E2" s="7">
-        <f t="shared" ref="E2:E28" si="0">IF(C2=0,0,+(C2-D2)/C2)</f>
+        <f t="shared" ref="E2:E29" si="0">IF(C2=0,0,+(C2-D2)/C2)</f>
         <v>0.63758389261744963</v>
       </c>
     </row>
@@ -1006,14 +1008,14 @@
         <v>39</v>
       </c>
       <c r="C21" s="6">
-        <v>0</v>
+        <v>96</v>
       </c>
       <c r="D21" s="6">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="E21" s="7">
         <f t="shared" ref="E21" si="1">IF(C21=0,0,+(C21-D21)/C21)</f>
-        <v>0</v>
+        <v>0.47916666666666669</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1048,34 +1050,34 @@
         <v>0</v>
       </c>
       <c r="E23" s="7">
-        <f t="shared" ref="E23" si="2">IF(C23=0,0,+(C23-D23)/C23)</f>
+        <f t="shared" ref="E23:E24" si="2">IF(C23=0,0,+(C23-D23)/C23)</f>
         <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="5">
-        <v>46298</v>
+      <c r="A24" s="10">
+        <v>46284</v>
       </c>
       <c r="B24" s="12" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="C24" s="6">
-        <v>0</v>
+        <v>363</v>
       </c>
       <c r="D24" s="6">
-        <v>0</v>
+        <v>163</v>
       </c>
       <c r="E24" s="7">
-        <f t="shared" si="0"/>
-        <v>0</v>
+        <f t="shared" si="2"/>
+        <v>0.55096418732782371</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="5">
-        <v>46319</v>
+        <v>46298</v>
       </c>
       <c r="B25" s="12" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C25" s="6">
         <v>0</v>
@@ -1093,7 +1095,7 @@
         <v>46319</v>
       </c>
       <c r="B26" s="12" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C26" s="6">
         <v>0</v>
@@ -1108,43 +1110,56 @@
     </row>
     <row r="27" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="5">
+        <v>46319</v>
+      </c>
+      <c r="B27" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="C27" s="6">
+        <v>0</v>
+      </c>
+      <c r="D27" s="6">
+        <v>0</v>
+      </c>
+      <c r="E27" s="7">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="5">
         <v>46333</v>
       </c>
-      <c r="B27" s="12" t="s">
+      <c r="B28" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="C27" s="6">
-        <v>0</v>
-      </c>
-      <c r="D27" s="6">
-        <v>0</v>
-      </c>
-      <c r="E27" s="7">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="5"/>
-      <c r="B28" s="12"/>
+      <c r="C28" s="6">
+        <v>0</v>
+      </c>
+      <c r="D28" s="6">
+        <v>0</v>
+      </c>
       <c r="E28" s="7">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="5"/>
       <c r="B29" s="12"/>
-      <c r="E29" s="7"/>
-    </row>
-    <row r="30" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E29" s="7">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="5"/>
-      <c r="B30" s="13"/>
+      <c r="B30" s="12"/>
       <c r="E30" s="7"/>
     </row>
     <row r="31" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="5"/>
-      <c r="B31" s="9"/>
+      <c r="B31" s="13"/>
       <c r="E31" s="7"/>
     </row>
     <row r="32" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1167,9 +1182,14 @@
       <c r="B35" s="9"/>
       <c r="E35" s="7"/>
     </row>
+    <row r="36" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="5"/>
+      <c r="B36" s="9"/>
+      <c r="E36" s="7"/>
+    </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I36">
-    <sortCondition ref="A2:A36"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I37">
+    <sortCondition ref="A2:A37"/>
   </sortState>
   <hyperlinks>
     <hyperlink ref="B2" r:id="rId1" display="https://sqlsaturday.com/2026-01-17-sqlsaturday1138/" xr:uid="{82BDF17B-780C-46C4-BDF3-6B50D2949365}"/>
@@ -1192,21 +1212,22 @@
     <hyperlink ref="B18" r:id="rId18" display="https://sqlsaturday.com/2026-07-18-sqlsaturday1141/" xr:uid="{B4310BB2-BE85-4D94-9531-7F04382A3C59}"/>
     <hyperlink ref="B19" r:id="rId19" display="https://sqlsaturday.com/2026-08-08-sqlsaturday1144/" xr:uid="{49013F68-7251-4303-A8A8-19F4C344B133}"/>
     <hyperlink ref="B22" r:id="rId20" display="https://sqlsaturday.com/2026-09-19-sqlsaturday1152/" xr:uid="{1C24212F-ACFE-4FD3-A6CF-8E691EEA9C75}"/>
-    <hyperlink ref="B24" r:id="rId21" display="https://sqlsaturday.com/2026-10-03-sqlsaturday1150/" xr:uid="{80072270-983F-4E6A-AFAE-3FC24DE448B3}"/>
-    <hyperlink ref="B25" r:id="rId22" display="https://sqlsaturday.com/2026-10-24-sqlsaturday1148/" xr:uid="{111A5B01-58C6-46AB-81AC-567A7B3C8861}"/>
-    <hyperlink ref="B26" r:id="rId23" display="https://sqlsaturday.com/2026-10-24-sqlsaturday1153/" xr:uid="{29A122E2-6150-4028-BEF4-E884CED9AA91}"/>
-    <hyperlink ref="B27" r:id="rId24" display="https://sqlsaturday.com/2026-11-07-sqlsaturday1149/" xr:uid="{1C87B471-8BB8-47E8-8A2F-FEB250EAF056}"/>
+    <hyperlink ref="B25" r:id="rId21" display="https://sqlsaturday.com/2026-10-03-sqlsaturday1150/" xr:uid="{80072270-983F-4E6A-AFAE-3FC24DE448B3}"/>
+    <hyperlink ref="B26" r:id="rId22" display="https://sqlsaturday.com/2026-10-24-sqlsaturday1148/" xr:uid="{111A5B01-58C6-46AB-81AC-567A7B3C8861}"/>
+    <hyperlink ref="B27" r:id="rId23" display="https://sqlsaturday.com/2026-10-24-sqlsaturday1153/" xr:uid="{29A122E2-6150-4028-BEF4-E884CED9AA91}"/>
+    <hyperlink ref="B28" r:id="rId24" display="https://sqlsaturday.com/2026-11-07-sqlsaturday1149/" xr:uid="{1C87B471-8BB8-47E8-8A2F-FEB250EAF056}"/>
     <hyperlink ref="B21" r:id="rId25" display="https://sqlsaturday.com/2026-09-12-sqlsaturday1164/" xr:uid="{C31C9E88-D474-46E9-9D7F-515DB0D1C4FD}"/>
     <hyperlink ref="B23" r:id="rId26" display="https://sqlsaturday.com/2026-09-19-sqlsaturday1156/" xr:uid="{D29C5250-03B6-490D-8B76-A7A1B304D760}"/>
+    <hyperlink ref="B24" r:id="rId27" display="https://sqlsaturday.com/2026-09-19-sqlsaturday1159/" xr:uid="{120DA250-32FF-4D5E-BAA0-AE998F27E101}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId27"/>
+  <pageSetup orientation="portrait" r:id="rId28"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C9FAEBE-70DD-4114-ACD9-DE4988A37B44}">
-  <dimension ref="A1:P29"/>
+  <dimension ref="A1:P30"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -1242,7 +1263,7 @@
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A2" s="24">
+      <c r="A2" s="10">
         <f>+Attendance!A2</f>
         <v>46039</v>
       </c>
@@ -1272,7 +1293,7 @@
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A3" s="24">
+      <c r="A3" s="10">
         <f>+Attendance!A3</f>
         <v>46102</v>
       </c>
@@ -1302,7 +1323,7 @@
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A4" s="24">
+      <c r="A4" s="10">
         <f>+Attendance!A4</f>
         <v>46109</v>
       </c>
@@ -1332,7 +1353,7 @@
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A5" s="24">
+      <c r="A5" s="10">
         <f>+Attendance!A5</f>
         <v>46123</v>
       </c>
@@ -1362,7 +1383,7 @@
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A6" s="24">
+      <c r="A6" s="10">
         <f>+Attendance!A6</f>
         <v>46123</v>
       </c>
@@ -1391,10 +1412,10 @@
         <v>167</v>
       </c>
       <c r="O6" s="20"/>
-      <c r="P6" s="23"/>
+      <c r="P6" s="24"/>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A7" s="24">
+      <c r="A7" s="10">
         <f>+Attendance!A7</f>
         <v>46130</v>
       </c>
@@ -1424,10 +1445,10 @@
         <v>134</v>
       </c>
       <c r="O7" s="21"/>
-      <c r="P7" s="23"/>
+      <c r="P7" s="24"/>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A8" s="24">
+      <c r="A8" s="10">
         <f>+Attendance!A8</f>
         <v>46137</v>
       </c>
@@ -1459,7 +1480,7 @@
       <c r="P8" s="22"/>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A9" s="24">
+      <c r="A9" s="10">
         <f>+Attendance!A9</f>
         <v>46137</v>
       </c>
@@ -1491,7 +1512,7 @@
       <c r="P9" s="22"/>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A10" s="24">
+      <c r="A10" s="10">
         <f>+Attendance!A10</f>
         <v>46144</v>
       </c>
@@ -1523,7 +1544,7 @@
       <c r="P10" s="22"/>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A11" s="24">
+      <c r="A11" s="10">
         <f>+Attendance!A11</f>
         <v>46158</v>
       </c>
@@ -1555,7 +1576,7 @@
       <c r="P11" s="22"/>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A12" s="24">
+      <c r="A12" s="10">
         <f>+Attendance!A12</f>
         <v>46256</v>
       </c>
@@ -1587,7 +1608,7 @@
       <c r="P12" s="22"/>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A13" s="24">
+      <c r="A13" s="10">
         <f>+Attendance!A13</f>
         <v>46165</v>
       </c>
@@ -1608,7 +1629,7 @@
         <v>0</v>
       </c>
       <c r="G13" s="8">
-        <f t="shared" ref="G13:G24" si="3">+H13-SUM(C13:F13)</f>
+        <f t="shared" ref="G13:G25" si="3">+H13-SUM(C13:F13)</f>
         <v>178</v>
       </c>
       <c r="H13" s="8">
@@ -1619,7 +1640,7 @@
       <c r="P13" s="22"/>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A14" s="24">
+      <c r="A14" s="10">
         <f>+Attendance!A14</f>
         <v>46172</v>
       </c>
@@ -1650,7 +1671,7 @@
       <c r="P14" s="22"/>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A15" s="24">
+      <c r="A15" s="10">
         <f>+Attendance!A15</f>
         <v>46186</v>
       </c>
@@ -1681,7 +1702,7 @@
       <c r="P15" s="22"/>
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A16" s="24">
+      <c r="A16" s="10">
         <f>+Attendance!A16</f>
         <v>46200</v>
       </c>
@@ -1712,7 +1733,7 @@
       <c r="P16" s="22"/>
     </row>
     <row r="17" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A17" s="24">
+      <c r="A17" s="10">
         <f>+Attendance!A17</f>
         <v>46200</v>
       </c>
@@ -1744,7 +1765,7 @@
       <c r="P17" s="22"/>
     </row>
     <row r="18" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A18" s="24">
+      <c r="A18" s="10">
         <f>+Attendance!A18</f>
         <v>46221</v>
       </c>
@@ -1776,7 +1797,7 @@
       <c r="P18" s="22"/>
     </row>
     <row r="19" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A19" s="24">
+      <c r="A19" s="10">
         <f>+Attendance!A19</f>
         <v>46242</v>
       </c>
@@ -1807,7 +1828,7 @@
       <c r="P19" s="22"/>
     </row>
     <row r="20" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A20" s="24">
+      <c r="A20" s="10">
         <f>+Attendance!A20</f>
         <v>46256</v>
       </c>
@@ -1839,67 +1860,67 @@
       <c r="P20" s="22"/>
     </row>
     <row r="21" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A21" s="25">
+      <c r="A21" s="23">
         <v>46277</v>
       </c>
       <c r="B21" s="12" t="s">
         <v>39</v>
       </c>
       <c r="C21">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="D21">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="E21">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F21">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="G21" s="8">
         <f t="shared" si="3"/>
+        <v>54</v>
+      </c>
+      <c r="H21" s="8">
+        <f>+Attendance!C21</f>
+        <v>96</v>
+      </c>
+      <c r="O21" s="21"/>
+      <c r="P21" s="22"/>
+    </row>
+    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A22" s="10">
+        <v>46284</v>
+      </c>
+      <c r="B22" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="C22">
+        <v>0</v>
+      </c>
+      <c r="D22">
+        <v>0</v>
+      </c>
+      <c r="E22">
+        <v>0</v>
+      </c>
+      <c r="F22">
+        <v>0</v>
+      </c>
+      <c r="G22" s="8">
+        <f t="shared" si="3"/>
         <v>140</v>
       </c>
-      <c r="H21" s="8">
+      <c r="H22" s="8">
         <f>+Attendance!C22</f>
         <v>140</v>
       </c>
-      <c r="O21" s="21"/>
-      <c r="P21" s="22"/>
-    </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A22" s="24">
-        <v>46284</v>
-      </c>
-      <c r="B22" s="12" t="s">
-        <v>34</v>
-      </c>
-      <c r="C22">
-        <v>0</v>
-      </c>
-      <c r="D22">
-        <v>0</v>
-      </c>
-      <c r="E22">
-        <v>0</v>
-      </c>
-      <c r="F22">
-        <v>0</v>
-      </c>
-      <c r="G22" s="8">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="H22" s="8">
-        <f>+Attendance!C24</f>
-        <v>0</v>
-      </c>
       <c r="O22" s="21"/>
       <c r="P22" s="22"/>
     </row>
     <row r="23" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A23" s="24">
+      <c r="A23" s="10">
         <v>46284</v>
       </c>
       <c r="B23" s="12" t="s">
@@ -1922,48 +1943,48 @@
         <v>0</v>
       </c>
       <c r="H23" s="8">
-        <f>+Attendance!C25</f>
+        <f>+Attendance!C23</f>
         <v>0</v>
       </c>
       <c r="O23" s="21"/>
       <c r="P23" s="22"/>
     </row>
     <row r="24" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A24" s="25">
-        <v>46298</v>
+      <c r="A24" s="10">
+        <v>46284</v>
       </c>
       <c r="B24" s="12" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="C24">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="D24">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E24">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F24">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="G24" s="8">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>324</v>
       </c>
       <c r="H24" s="8">
-        <f>+Attendance!C26</f>
-        <v>0</v>
+        <f>+Attendance!C24</f>
+        <v>363</v>
       </c>
       <c r="O24" s="21"/>
       <c r="P24" s="22"/>
     </row>
     <row r="25" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A25" s="25">
-        <v>46319</v>
+      <c r="A25" s="23">
+        <v>46298</v>
       </c>
       <c r="B25" s="12" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C25">
         <v>0</v>
@@ -1978,22 +1999,22 @@
         <v>0</v>
       </c>
       <c r="G25" s="8">
-        <f t="shared" ref="G25" si="4">+H25-SUM(C25:F25)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="H25" s="8">
-        <f>+Attendance!C27</f>
+        <f>+Attendance!C25</f>
         <v>0</v>
       </c>
       <c r="O25" s="21"/>
       <c r="P25" s="22"/>
     </row>
     <row r="26" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A26" s="25">
+      <c r="A26" s="23">
         <v>46319</v>
       </c>
       <c r="B26" s="12" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C26">
         <v>0</v>
@@ -2008,22 +2029,22 @@
         <v>0</v>
       </c>
       <c r="G26" s="8">
-        <f t="shared" ref="G26:G27" si="5">+H26-SUM(C26:F26)</f>
+        <f t="shared" ref="G26" si="4">+H26-SUM(C26:F26)</f>
         <v>0</v>
       </c>
       <c r="H26" s="8">
-        <f>+Attendance!C28</f>
+        <f>+Attendance!C26</f>
         <v>0</v>
       </c>
       <c r="O26" s="21"/>
       <c r="P26" s="22"/>
     </row>
     <row r="27" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A27" s="25">
-        <v>46333</v>
+      <c r="A27" s="23">
+        <v>46319</v>
       </c>
       <c r="B27" s="12" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C27">
         <v>0</v>
@@ -2038,23 +2059,53 @@
         <v>0</v>
       </c>
       <c r="G27" s="8">
-        <f t="shared" si="5"/>
+        <f t="shared" ref="G27:G28" si="5">+H27-SUM(C27:F27)</f>
         <v>0</v>
       </c>
       <c r="H27" s="8">
-        <f>+Attendance!C29</f>
+        <f>+Attendance!C27</f>
         <v>0</v>
       </c>
       <c r="O27" s="21"/>
       <c r="P27" s="22"/>
     </row>
     <row r="28" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A28" s="23">
+        <v>46333</v>
+      </c>
+      <c r="B28" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="C28">
+        <v>0</v>
+      </c>
+      <c r="D28">
+        <v>0</v>
+      </c>
+      <c r="E28">
+        <v>0</v>
+      </c>
+      <c r="F28">
+        <v>0</v>
+      </c>
+      <c r="G28" s="8">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="H28" s="8">
+        <f>+Attendance!C28</f>
+        <v>0</v>
+      </c>
       <c r="O28" s="21"/>
       <c r="P28" s="22"/>
     </row>
     <row r="29" spans="1:16" x14ac:dyDescent="0.25">
       <c r="O29" s="21"/>
       <c r="P29" s="22"/>
+    </row>
+    <row r="30" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="O30" s="21"/>
+      <c r="P30" s="22"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2062,14 +2113,15 @@
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="B22" r:id="rId1" display="https://sqlsaturday.com/2026-09-19-sqlsaturday1152/" xr:uid="{0D6A567B-FCB7-44A2-A51E-648C719A8354}"/>
-    <hyperlink ref="B24" r:id="rId2" display="https://sqlsaturday.com/2026-10-03-sqlsaturday1150/" xr:uid="{D31F3CEB-8FBE-4CA1-97BB-2A40A92A8401}"/>
-    <hyperlink ref="B25" r:id="rId3" display="https://sqlsaturday.com/2026-10-24-sqlsaturday1148/" xr:uid="{96299D66-5563-46A3-B76A-F680ABDD2206}"/>
-    <hyperlink ref="B26" r:id="rId4" display="https://sqlsaturday.com/2026-10-24-sqlsaturday1153/" xr:uid="{4FAC5D40-7DBE-4A53-AFF9-C92E65F31759}"/>
-    <hyperlink ref="B27" r:id="rId5" display="https://sqlsaturday.com/2026-11-07-sqlsaturday1149/" xr:uid="{45E94655-95AF-4485-A5A2-4A3DD7455E27}"/>
+    <hyperlink ref="B25" r:id="rId2" display="https://sqlsaturday.com/2026-10-03-sqlsaturday1150/" xr:uid="{D31F3CEB-8FBE-4CA1-97BB-2A40A92A8401}"/>
+    <hyperlink ref="B26" r:id="rId3" display="https://sqlsaturday.com/2026-10-24-sqlsaturday1148/" xr:uid="{96299D66-5563-46A3-B76A-F680ABDD2206}"/>
+    <hyperlink ref="B27" r:id="rId4" display="https://sqlsaturday.com/2026-10-24-sqlsaturday1153/" xr:uid="{4FAC5D40-7DBE-4A53-AFF9-C92E65F31759}"/>
+    <hyperlink ref="B28" r:id="rId5" display="https://sqlsaturday.com/2026-11-07-sqlsaturday1149/" xr:uid="{45E94655-95AF-4485-A5A2-4A3DD7455E27}"/>
     <hyperlink ref="B21" r:id="rId6" display="https://sqlsaturday.com/2026-09-12-sqlsaturday1164/" xr:uid="{5E7F8464-7EFE-4379-AF7A-413F4F14ABD5}"/>
     <hyperlink ref="B23" r:id="rId7" display="https://sqlsaturday.com/2026-09-19-sqlsaturday1156/" xr:uid="{840B9723-899E-4E77-BBFA-21BF1FA89943}"/>
+    <hyperlink ref="B24" r:id="rId8" display="https://sqlsaturday.com/2026-09-19-sqlsaturday1159/" xr:uid="{0795C785-E600-4CBB-BC80-E9889F632DF8}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId8"/>
+  <pageSetup orientation="portrait" r:id="rId9"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Toronto, Floripa updates (#1436)
* Toronto, Floripa updates

* release ATL date

* remove past events

---------

Co-authored-by: way0utwest <admin@sqlsaturday.com>
</commit_message>
<xml_diff>
--- a/assets/misc/2026/2026_Attendance.xlsx
+++ b/assets/misc/2026/2026_Attendance.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Documents\git\sqlsatwebsite\assets\misc\2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D96B25A-5DA8-4948-B5A1-87C51D0AB38E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF042CDF-35DF-4E93-83C5-5214A96456C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28245" yWindow="315" windowWidth="25260" windowHeight="15210" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-25695" yWindow="75" windowWidth="25260" windowHeight="15210" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Attendance" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="45">
   <si>
     <t>Date</t>
   </si>
@@ -160,6 +160,15 @@
   </si>
   <si>
     <t>Day of Data Winnipeg 2026 (#1159)</t>
+  </si>
+  <si>
+    <t>SQL Saturday Floripa 2026 (#1158)</t>
+  </si>
+  <si>
+    <t>Day of Data Orlando 2026 (#1161)</t>
+  </si>
+  <si>
+    <t>Day of Data Toronto 2026 (#1160)</t>
   </si>
 </sst>
 </file>
@@ -615,7 +624,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:I36"/>
+  <dimension ref="A1:I39"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.7109375" style="10" bestFit="1" customWidth="1"/>
@@ -669,7 +678,7 @@
         <v>108</v>
       </c>
       <c r="E2" s="7">
-        <f t="shared" ref="E2:E29" si="0">IF(C2=0,0,+(C2-D2)/C2)</f>
+        <f t="shared" ref="E2:E32" si="0">IF(C2=0,0,+(C2-D2)/C2)</f>
         <v>0.63758389261744963</v>
       </c>
     </row>
@@ -1050,7 +1059,7 @@
         <v>376</v>
       </c>
       <c r="E23" s="7">
-        <f t="shared" ref="E23:E24" si="2">IF(C23=0,0,+(C23-D23)/C23)</f>
+        <f t="shared" ref="E23:E25" si="2">IF(C23=0,0,+(C23-D23)/C23)</f>
         <v>0.70039840637450201</v>
       </c>
     </row>
@@ -1073,108 +1082,147 @@
       </c>
     </row>
     <row r="25" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="5">
-        <v>46298</v>
+      <c r="A25" s="10">
+        <v>46291</v>
       </c>
       <c r="B25" s="12" t="s">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="C25" s="6">
-        <v>226</v>
+        <v>320</v>
       </c>
       <c r="D25" s="6">
-        <v>176</v>
+        <v>249</v>
       </c>
       <c r="E25" s="7">
-        <f t="shared" si="0"/>
-        <v>0.22123893805309736</v>
+        <f t="shared" si="2"/>
+        <v>0.22187499999999999</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="5">
+        <v>46298</v>
+      </c>
+      <c r="B26" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="C26" s="6">
+        <v>226</v>
+      </c>
+      <c r="D26" s="6">
+        <v>176</v>
+      </c>
+      <c r="E26" s="7">
+        <f t="shared" si="0"/>
+        <v>0.22123893805309736</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="23">
+        <v>46305</v>
+      </c>
+      <c r="B27" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="C27" s="6">
+        <v>0</v>
+      </c>
+      <c r="D27" s="6">
+        <v>0</v>
+      </c>
+      <c r="E27" s="7">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="23">
+        <v>46305</v>
+      </c>
+      <c r="B28" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="C28" s="6">
+        <v>200</v>
+      </c>
+      <c r="D28" s="6">
+        <v>100</v>
+      </c>
+      <c r="E28" s="7">
+        <f t="shared" si="0"/>
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="5">
         <v>46319</v>
       </c>
-      <c r="B26" s="12" t="s">
+      <c r="B29" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="C26" s="6">
-        <v>0</v>
-      </c>
-      <c r="D26" s="6">
-        <v>0</v>
-      </c>
-      <c r="E26" s="7">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="5">
+      <c r="C29" s="6">
+        <v>0</v>
+      </c>
+      <c r="D29" s="6">
+        <v>0</v>
+      </c>
+      <c r="E29" s="7">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="5">
         <v>46319</v>
       </c>
-      <c r="B27" s="12" t="s">
+      <c r="B30" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="C27" s="6">
-        <v>0</v>
-      </c>
-      <c r="D27" s="6">
-        <v>0</v>
-      </c>
-      <c r="E27" s="7">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="5">
+      <c r="C30" s="6">
+        <v>0</v>
+      </c>
+      <c r="D30" s="6">
+        <v>0</v>
+      </c>
+      <c r="E30" s="7">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="5">
         <v>46333</v>
       </c>
-      <c r="B28" s="12" t="s">
+      <c r="B31" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="C28" s="6">
-        <v>0</v>
-      </c>
-      <c r="D28" s="6">
-        <v>0</v>
-      </c>
-      <c r="E28" s="7">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="5"/>
-      <c r="B29" s="12"/>
-      <c r="E29" s="7">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="5"/>
-      <c r="B30" s="12"/>
-      <c r="E30" s="7"/>
-    </row>
-    <row r="31" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="5"/>
-      <c r="B31" s="13"/>
-      <c r="E31" s="7"/>
+      <c r="C31" s="6">
+        <v>0</v>
+      </c>
+      <c r="D31" s="6">
+        <v>0</v>
+      </c>
+      <c r="E31" s="7">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="32" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="5"/>
-      <c r="B32" s="9"/>
-      <c r="E32" s="7"/>
-    </row>
-    <row r="33" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B32" s="12"/>
+      <c r="E32" s="7">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="5"/>
-      <c r="B33" s="9"/>
+      <c r="B33" s="12"/>
       <c r="E33" s="7"/>
     </row>
     <row r="34" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="5"/>
-      <c r="B34" s="9"/>
+      <c r="B34" s="13"/>
       <c r="E34" s="7"/>
     </row>
     <row r="35" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1187,9 +1235,24 @@
       <c r="B36" s="9"/>
       <c r="E36" s="7"/>
     </row>
+    <row r="37" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="5"/>
+      <c r="B37" s="9"/>
+      <c r="E37" s="7"/>
+    </row>
+    <row r="38" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="5"/>
+      <c r="B38" s="9"/>
+      <c r="E38" s="7"/>
+    </row>
+    <row r="39" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="5"/>
+      <c r="B39" s="9"/>
+      <c r="E39" s="7"/>
+    </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I37">
-    <sortCondition ref="A2:A37"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I40">
+    <sortCondition ref="A2:A40"/>
   </sortState>
   <hyperlinks>
     <hyperlink ref="B2" r:id="rId1" display="https://sqlsaturday.com/2026-01-17-sqlsaturday1138/" xr:uid="{82BDF17B-780C-46C4-BDF3-6B50D2949365}"/>
@@ -1212,22 +1275,25 @@
     <hyperlink ref="B18" r:id="rId18" display="https://sqlsaturday.com/2026-07-18-sqlsaturday1141/" xr:uid="{B4310BB2-BE85-4D94-9531-7F04382A3C59}"/>
     <hyperlink ref="B19" r:id="rId19" display="https://sqlsaturday.com/2026-08-08-sqlsaturday1144/" xr:uid="{49013F68-7251-4303-A8A8-19F4C344B133}"/>
     <hyperlink ref="B22" r:id="rId20" display="https://sqlsaturday.com/2026-09-19-sqlsaturday1152/" xr:uid="{1C24212F-ACFE-4FD3-A6CF-8E691EEA9C75}"/>
-    <hyperlink ref="B25" r:id="rId21" display="https://sqlsaturday.com/2026-10-03-sqlsaturday1150/" xr:uid="{80072270-983F-4E6A-AFAE-3FC24DE448B3}"/>
-    <hyperlink ref="B26" r:id="rId22" display="https://sqlsaturday.com/2026-10-24-sqlsaturday1148/" xr:uid="{111A5B01-58C6-46AB-81AC-567A7B3C8861}"/>
-    <hyperlink ref="B27" r:id="rId23" display="https://sqlsaturday.com/2026-10-24-sqlsaturday1153/" xr:uid="{29A122E2-6150-4028-BEF4-E884CED9AA91}"/>
-    <hyperlink ref="B28" r:id="rId24" display="https://sqlsaturday.com/2026-11-07-sqlsaturday1149/" xr:uid="{1C87B471-8BB8-47E8-8A2F-FEB250EAF056}"/>
+    <hyperlink ref="B26" r:id="rId21" display="https://sqlsaturday.com/2026-10-03-sqlsaturday1150/" xr:uid="{80072270-983F-4E6A-AFAE-3FC24DE448B3}"/>
+    <hyperlink ref="B29" r:id="rId22" display="https://sqlsaturday.com/2026-10-24-sqlsaturday1148/" xr:uid="{111A5B01-58C6-46AB-81AC-567A7B3C8861}"/>
+    <hyperlink ref="B30" r:id="rId23" display="https://sqlsaturday.com/2026-10-24-sqlsaturday1153/" xr:uid="{29A122E2-6150-4028-BEF4-E884CED9AA91}"/>
+    <hyperlink ref="B31" r:id="rId24" display="https://sqlsaturday.com/2026-11-07-sqlsaturday1149/" xr:uid="{1C87B471-8BB8-47E8-8A2F-FEB250EAF056}"/>
     <hyperlink ref="B21" r:id="rId25" display="https://sqlsaturday.com/2026-09-12-sqlsaturday1164/" xr:uid="{C31C9E88-D474-46E9-9D7F-515DB0D1C4FD}"/>
     <hyperlink ref="B23" r:id="rId26" display="https://sqlsaturday.com/2026-09-19-sqlsaturday1156/" xr:uid="{D29C5250-03B6-490D-8B76-A7A1B304D760}"/>
     <hyperlink ref="B24" r:id="rId27" display="https://sqlsaturday.com/2026-09-19-sqlsaturday1159/" xr:uid="{120DA250-32FF-4D5E-BAA0-AE998F27E101}"/>
+    <hyperlink ref="B28" r:id="rId28" display="https://sqlsaturday.com/2026-10-17-sqlsaturday1158/" xr:uid="{2D6CCE83-4261-41C0-B4C4-43B0C3FABEA6}"/>
+    <hyperlink ref="B27" r:id="rId29" display="https://sqlsaturday.com/2026-10-17-sqlsaturday1161/" xr:uid="{4A13ED3F-D3DC-400D-9262-574D23DDA0BF}"/>
+    <hyperlink ref="B25" r:id="rId30" display="https://sqlsaturday.com/2026-09-26-sqlsaturday1160/" xr:uid="{CF95E3B9-8C45-4ACB-9719-85DEDE16399E}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId28"/>
+  <pageSetup orientation="portrait" r:id="rId31"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C9FAEBE-70DD-4114-ACD9-DE4988A37B44}">
-  <dimension ref="A1:P30"/>
+  <dimension ref="A1:P34"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -1629,7 +1695,7 @@
         <v>0</v>
       </c>
       <c r="G13" s="8">
-        <f t="shared" ref="G13:G25" si="3">+H13-SUM(C13:F13)</f>
+        <f t="shared" ref="G13:G27" si="3">+H13-SUM(C13:F13)</f>
         <v>178</v>
       </c>
       <c r="H13" s="8">
@@ -1980,71 +2046,71 @@
       <c r="P24" s="22"/>
     </row>
     <row r="25" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A25" s="23">
+      <c r="A25" s="10">
+        <v>46291</v>
+      </c>
+      <c r="B25" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="C25">
+        <v>21</v>
+      </c>
+      <c r="D25">
+        <v>15</v>
+      </c>
+      <c r="E25">
+        <v>7</v>
+      </c>
+      <c r="F25">
+        <v>38</v>
+      </c>
+      <c r="G25" s="8">
+        <f t="shared" ref="G25" si="4">+H25-SUM(C25:F25)</f>
+        <v>239</v>
+      </c>
+      <c r="H25" s="8">
+        <f>+Attendance!C25</f>
+        <v>320</v>
+      </c>
+      <c r="O25" s="21"/>
+      <c r="P25" s="22"/>
+    </row>
+    <row r="26" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A26" s="23">
         <v>46298</v>
       </c>
-      <c r="B25" s="12" t="s">
+      <c r="B26" s="12" t="s">
         <v>35</v>
       </c>
-      <c r="C25">
-        <v>0</v>
-      </c>
-      <c r="D25">
-        <v>0</v>
-      </c>
-      <c r="E25">
-        <v>0</v>
-      </c>
-      <c r="F25">
-        <v>0</v>
-      </c>
-      <c r="G25" s="8">
+      <c r="C26">
+        <v>0</v>
+      </c>
+      <c r="D26">
+        <v>0</v>
+      </c>
+      <c r="E26">
+        <v>0</v>
+      </c>
+      <c r="F26">
+        <v>0</v>
+      </c>
+      <c r="G26" s="8">
         <f t="shared" si="3"/>
         <v>226</v>
       </c>
-      <c r="H25" s="8">
-        <f>+Attendance!C25</f>
-        <v>226</v>
-      </c>
-      <c r="O25" s="21"/>
-      <c r="P25" s="22"/>
-    </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A26" s="23">
-        <v>46319</v>
-      </c>
-      <c r="B26" s="12" t="s">
-        <v>36</v>
-      </c>
-      <c r="C26">
-        <v>0</v>
-      </c>
-      <c r="D26">
-        <v>0</v>
-      </c>
-      <c r="E26">
-        <v>0</v>
-      </c>
-      <c r="F26">
-        <v>0</v>
-      </c>
-      <c r="G26" s="8">
-        <f t="shared" ref="G26" si="4">+H26-SUM(C26:F26)</f>
-        <v>0</v>
-      </c>
       <c r="H26" s="8">
         <f>+Attendance!C26</f>
-        <v>0</v>
+        <v>226</v>
       </c>
       <c r="O26" s="21"/>
       <c r="P26" s="22"/>
     </row>
     <row r="27" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A27" s="23">
-        <v>46319</v>
+        <v>46305</v>
       </c>
       <c r="B27" s="12" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="C27">
         <v>0</v>
@@ -2059,22 +2125,22 @@
         <v>0</v>
       </c>
       <c r="G27" s="8">
-        <f t="shared" ref="G27:G28" si="5">+H27-SUM(C27:F27)</f>
-        <v>0</v>
+        <f t="shared" si="3"/>
+        <v>363</v>
       </c>
       <c r="H27" s="8">
-        <f>+Attendance!C27</f>
-        <v>0</v>
+        <f>+Attendance!C24</f>
+        <v>363</v>
       </c>
       <c r="O27" s="21"/>
       <c r="P27" s="22"/>
     </row>
     <row r="28" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A28" s="23">
-        <v>46333</v>
+        <v>46305</v>
       </c>
       <c r="B28" s="12" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="C28">
         <v>0</v>
@@ -2089,23 +2155,143 @@
         <v>0</v>
       </c>
       <c r="G28" s="8">
-        <f t="shared" si="5"/>
-        <v>0</v>
+        <f t="shared" ref="G28" si="5">+H28-SUM(C28:F28)</f>
+        <v>226</v>
       </c>
       <c r="H28" s="8">
-        <f>+Attendance!C28</f>
-        <v>0</v>
+        <f>+Attendance!C26</f>
+        <v>226</v>
       </c>
       <c r="O28" s="21"/>
       <c r="P28" s="22"/>
     </row>
     <row r="29" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A29" s="23">
+        <v>46312</v>
+      </c>
+      <c r="B29" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="C29">
+        <v>0</v>
+      </c>
+      <c r="D29">
+        <v>0</v>
+      </c>
+      <c r="E29">
+        <v>0</v>
+      </c>
+      <c r="F29">
+        <v>0</v>
+      </c>
+      <c r="G29" s="8">
+        <f t="shared" ref="G29" si="6">+H29-SUM(C29:F29)</f>
+        <v>0</v>
+      </c>
+      <c r="H29" s="8">
+        <f>+Attendance!C29</f>
+        <v>0</v>
+      </c>
       <c r="O29" s="21"/>
       <c r="P29" s="22"/>
     </row>
     <row r="30" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A30" s="23">
+        <v>46319</v>
+      </c>
+      <c r="B30" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="C30">
+        <v>0</v>
+      </c>
+      <c r="D30">
+        <v>0</v>
+      </c>
+      <c r="E30">
+        <v>0</v>
+      </c>
+      <c r="F30">
+        <v>0</v>
+      </c>
+      <c r="G30" s="8">
+        <f t="shared" ref="G30" si="7">+H30-SUM(C30:F30)</f>
+        <v>0</v>
+      </c>
+      <c r="H30" s="8">
+        <f>+Attendance!C29</f>
+        <v>0</v>
+      </c>
       <c r="O30" s="21"/>
       <c r="P30" s="22"/>
+    </row>
+    <row r="31" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A31" s="23">
+        <v>46319</v>
+      </c>
+      <c r="B31" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="C31">
+        <v>0</v>
+      </c>
+      <c r="D31">
+        <v>0</v>
+      </c>
+      <c r="E31">
+        <v>0</v>
+      </c>
+      <c r="F31">
+        <v>0</v>
+      </c>
+      <c r="G31" s="8">
+        <f t="shared" ref="G31:G32" si="8">+H31-SUM(C31:F31)</f>
+        <v>0</v>
+      </c>
+      <c r="H31" s="8">
+        <f>+Attendance!C30</f>
+        <v>0</v>
+      </c>
+      <c r="O31" s="21"/>
+      <c r="P31" s="22"/>
+    </row>
+    <row r="32" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A32" s="23">
+        <v>46333</v>
+      </c>
+      <c r="B32" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="C32">
+        <v>0</v>
+      </c>
+      <c r="D32">
+        <v>0</v>
+      </c>
+      <c r="E32">
+        <v>0</v>
+      </c>
+      <c r="F32">
+        <v>0</v>
+      </c>
+      <c r="G32" s="8">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="H32" s="8">
+        <f>+Attendance!C31</f>
+        <v>0</v>
+      </c>
+      <c r="O32" s="21"/>
+      <c r="P32" s="22"/>
+    </row>
+    <row r="33" spans="15:16" x14ac:dyDescent="0.25">
+      <c r="O33" s="21"/>
+      <c r="P33" s="22"/>
+    </row>
+    <row r="34" spans="15:16" x14ac:dyDescent="0.25">
+      <c r="O34" s="21"/>
+      <c r="P34" s="22"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2113,15 +2299,19 @@
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="B22" r:id="rId1" display="https://sqlsaturday.com/2026-09-19-sqlsaturday1152/" xr:uid="{0D6A567B-FCB7-44A2-A51E-648C719A8354}"/>
-    <hyperlink ref="B25" r:id="rId2" display="https://sqlsaturday.com/2026-10-03-sqlsaturday1150/" xr:uid="{D31F3CEB-8FBE-4CA1-97BB-2A40A92A8401}"/>
-    <hyperlink ref="B26" r:id="rId3" display="https://sqlsaturday.com/2026-10-24-sqlsaturday1148/" xr:uid="{96299D66-5563-46A3-B76A-F680ABDD2206}"/>
-    <hyperlink ref="B27" r:id="rId4" display="https://sqlsaturday.com/2026-10-24-sqlsaturday1153/" xr:uid="{4FAC5D40-7DBE-4A53-AFF9-C92E65F31759}"/>
-    <hyperlink ref="B28" r:id="rId5" display="https://sqlsaturday.com/2026-11-07-sqlsaturday1149/" xr:uid="{45E94655-95AF-4485-A5A2-4A3DD7455E27}"/>
+    <hyperlink ref="B26" r:id="rId2" display="https://sqlsaturday.com/2026-10-03-sqlsaturday1150/" xr:uid="{D31F3CEB-8FBE-4CA1-97BB-2A40A92A8401}"/>
+    <hyperlink ref="B30" r:id="rId3" display="https://sqlsaturday.com/2026-10-24-sqlsaturday1148/" xr:uid="{96299D66-5563-46A3-B76A-F680ABDD2206}"/>
+    <hyperlink ref="B31" r:id="rId4" display="https://sqlsaturday.com/2026-10-24-sqlsaturday1153/" xr:uid="{4FAC5D40-7DBE-4A53-AFF9-C92E65F31759}"/>
+    <hyperlink ref="B32" r:id="rId5" display="https://sqlsaturday.com/2026-11-07-sqlsaturday1149/" xr:uid="{45E94655-95AF-4485-A5A2-4A3DD7455E27}"/>
     <hyperlink ref="B21" r:id="rId6" display="https://sqlsaturday.com/2026-09-12-sqlsaturday1164/" xr:uid="{5E7F8464-7EFE-4379-AF7A-413F4F14ABD5}"/>
     <hyperlink ref="B23" r:id="rId7" display="https://sqlsaturday.com/2026-09-19-sqlsaturday1156/" xr:uid="{840B9723-899E-4E77-BBFA-21BF1FA89943}"/>
     <hyperlink ref="B24" r:id="rId8" display="https://sqlsaturday.com/2026-09-19-sqlsaturday1159/" xr:uid="{0795C785-E600-4CBB-BC80-E9889F632DF8}"/>
+    <hyperlink ref="B29" r:id="rId9" display="https://sqlsaturday.com/2026-10-17-sqlsaturday1158/" xr:uid="{C525B75A-FA66-455E-9044-8EAD66B8FD62}"/>
+    <hyperlink ref="B28" r:id="rId10" display="https://sqlsaturday.com/2026-10-17-sqlsaturday1158/" xr:uid="{5E334D9F-9799-4B32-A293-64E5718D75C1}"/>
+    <hyperlink ref="B27" r:id="rId11" display="https://sqlsaturday.com/2026-10-17-sqlsaturday1161/" xr:uid="{83C5546A-C2FB-4A01-A556-E429A4F7B664}"/>
+    <hyperlink ref="B25" r:id="rId12" display="https://sqlsaturday.com/2026-09-26-sqlsaturday1160/" xr:uid="{C805518F-632E-48E7-AEE4-3AFAF9705381}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId9"/>
+  <pageSetup orientation="portrait" r:id="rId13"/>
 </worksheet>
 </file>
</xml_diff>